<commit_message>
auto update Sun 05/31/2026 14:12:51.74
</commit_message>
<xml_diff>
--- a/WagonsWithWeight.xlsx
+++ b/WagonsWithWeight.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HAISB STORE\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1B519618-0A01-45F4-9686-90CD114CF0F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8578473-0519-4183-A337-97FAE5671AE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{68AA4FA8-561F-47EB-AC86-75E02A3E7FE4}"/>
+    <workbookView xWindow="8190" yWindow="1125" windowWidth="21600" windowHeight="11235" xr2:uid="{68AA4FA8-561F-47EB-AC86-75E02A3E7FE4}"/>
   </bookViews>
   <sheets>
     <sheet name="WagonsWithWeight" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5075" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5138" uniqueCount="103">
   <si>
     <t>تاریخ</t>
   </si>
@@ -918,6 +918,7 @@
       <sheetName val="master table"/>
       <sheetName val="mater tabel for tracks"/>
       <sheetName val="WagonsWithWeight"/>
+      <sheetName val="Sheet3"/>
       <sheetName val="FinancialStatement"/>
       <sheetName val="Data Source"/>
       <sheetName val="source"/>
@@ -939,6 +940,7 @@
       <sheetData sheetId="8"/>
       <sheetData sheetId="9"/>
       <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1010,7 +1012,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7A8B5CD-448E-48E3-8458-B8CC5030BD56}" name="Table6" displayName="Table6" ref="A1:H1690" headerRowDxfId="20" dataDxfId="19" headerRowBorderDxfId="17" tableBorderDxfId="18" totalsRowBorderDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7A8B5CD-448E-48E3-8458-B8CC5030BD56}" name="Table6" displayName="Table6" ref="A1:H1711" headerRowDxfId="20" dataDxfId="19" headerRowBorderDxfId="17" tableBorderDxfId="18" totalsRowBorderDxfId="16">
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H1340">
     <sortCondition ref="A1:A1340"/>
   </sortState>
@@ -1326,7 +1328,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26D80CA6-9C60-4A13-87BC-5BF4E6FD5B80}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:H1690"/>
+  <dimension ref="A1:H1711"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" style="11" bestFit="1" customWidth="1"/>
@@ -45279,6 +45281,510 @@
         <v>3</v>
       </c>
     </row>
+    <row r="1691" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1691" s="5">
+        <v>46165</v>
+      </c>
+      <c r="B1691" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1691" s="6">
+        <v>28848133</v>
+      </c>
+      <c r="D1691" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1691" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1691" s="6">
+        <v>1359</v>
+      </c>
+      <c r="G1691" s="6">
+        <v>67950</v>
+      </c>
+      <c r="H1691" s="7"/>
+    </row>
+    <row r="1692" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1692" s="5">
+        <v>46165</v>
+      </c>
+      <c r="B1692" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1692" s="6">
+        <v>28090264</v>
+      </c>
+      <c r="D1692" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1692" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1692" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1692" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1692" s="7"/>
+    </row>
+    <row r="1693" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1693" s="5">
+        <v>46165</v>
+      </c>
+      <c r="B1693" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1693" s="6">
+        <v>28090785</v>
+      </c>
+      <c r="D1693" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1693" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1693" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1693" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1693" s="7"/>
+    </row>
+    <row r="1694" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1694" s="5">
+        <v>46165</v>
+      </c>
+      <c r="B1694" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1694" s="6">
+        <v>28847770</v>
+      </c>
+      <c r="D1694" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1694" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1694" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1694" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1694" s="7"/>
+    </row>
+    <row r="1695" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1695" s="5">
+        <v>46165</v>
+      </c>
+      <c r="B1695" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1695" s="6">
+        <v>28846830</v>
+      </c>
+      <c r="D1695" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1695" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1695" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1695" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1695" s="7"/>
+    </row>
+    <row r="1696" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1696" s="5">
+        <v>46166</v>
+      </c>
+      <c r="B1696" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1696" s="6">
+        <v>29021144</v>
+      </c>
+      <c r="D1696" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1696" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1696" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1696" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1696" s="7"/>
+    </row>
+    <row r="1697" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1697" s="5">
+        <v>46166</v>
+      </c>
+      <c r="B1697" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1697" s="6">
+        <v>28002517</v>
+      </c>
+      <c r="D1697" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1697" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1697" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1697" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1697" s="7"/>
+    </row>
+    <row r="1698" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1698" s="5">
+        <v>46166</v>
+      </c>
+      <c r="B1698" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1698" s="6">
+        <v>29840592</v>
+      </c>
+      <c r="D1698" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1698" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1698" s="6">
+        <v>1340</v>
+      </c>
+      <c r="G1698" s="6">
+        <v>67000</v>
+      </c>
+      <c r="H1698" s="7"/>
+    </row>
+    <row r="1699" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1699" s="5">
+        <v>46166</v>
+      </c>
+      <c r="B1699" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1699" s="6">
+        <v>28855153</v>
+      </c>
+      <c r="D1699" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1699" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1699" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1699" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1699" s="7"/>
+    </row>
+    <row r="1700" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1700" s="5">
+        <v>46166</v>
+      </c>
+      <c r="B1700" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1700" s="6">
+        <v>28856086</v>
+      </c>
+      <c r="D1700" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1700" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1700" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1700" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1700" s="7"/>
+    </row>
+    <row r="1701" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1701" s="5">
+        <v>46166</v>
+      </c>
+      <c r="B1701" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1701" s="6">
+        <v>28854131</v>
+      </c>
+      <c r="D1701" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1701" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1701" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1701" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1701" s="7"/>
+    </row>
+    <row r="1702" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1702" s="5">
+        <v>46166</v>
+      </c>
+      <c r="B1702" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1702" s="6">
+        <v>28856144</v>
+      </c>
+      <c r="D1702" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1702" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1702" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1702" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1702" s="7"/>
+    </row>
+    <row r="1703" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1703" s="5">
+        <v>46166</v>
+      </c>
+      <c r="B1703" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1703" s="6">
+        <v>28856029</v>
+      </c>
+      <c r="D1703" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1703" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1703" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1703" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1703" s="7"/>
+    </row>
+    <row r="1704" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1704" s="5">
+        <v>46167</v>
+      </c>
+      <c r="B1704" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1704" s="6">
+        <v>29221074</v>
+      </c>
+      <c r="D1704" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1704" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1704" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1704" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1704" s="7"/>
+    </row>
+    <row r="1705" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1705" s="5">
+        <v>46167</v>
+      </c>
+      <c r="B1705" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1705" s="6">
+        <v>29410305</v>
+      </c>
+      <c r="D1705" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1705" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1705" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1705" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1705" s="7"/>
+    </row>
+    <row r="1706" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1706" s="5">
+        <v>46167</v>
+      </c>
+      <c r="B1706" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1706" s="6">
+        <v>29135431</v>
+      </c>
+      <c r="D1706" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1706" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1706" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1706" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1706" s="7"/>
+    </row>
+    <row r="1707" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1707" s="5">
+        <v>46167</v>
+      </c>
+      <c r="B1707" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1707" s="6">
+        <v>29221009</v>
+      </c>
+      <c r="D1707" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1707" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1707" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1707" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1707" s="7"/>
+    </row>
+    <row r="1708" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1708" s="5">
+        <v>46167</v>
+      </c>
+      <c r="B1708" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1708" s="6">
+        <v>28819480</v>
+      </c>
+      <c r="D1708" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1708" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1708" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1708" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1708" s="7"/>
+    </row>
+    <row r="1709" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1709" s="5">
+        <v>46167</v>
+      </c>
+      <c r="B1709" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1709" s="6">
+        <v>28349660</v>
+      </c>
+      <c r="D1709" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1709" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1709" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1709" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1709" s="7"/>
+    </row>
+    <row r="1710" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1710" s="5">
+        <v>46167</v>
+      </c>
+      <c r="B1710" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1710" s="6">
+        <v>28026961</v>
+      </c>
+      <c r="D1710" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1710" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1710" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1710" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1710" s="7"/>
+    </row>
+    <row r="1711" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1711" s="8">
+        <v>46166</v>
+      </c>
+      <c r="B1711" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1711" s="9">
+        <v>91138644</v>
+      </c>
+      <c r="D1711" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1711" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F1711" s="9">
+        <v>1303</v>
+      </c>
+      <c r="G1711" s="9">
+        <v>68100</v>
+      </c>
+      <c r="H1711" s="10"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
auto update Sun 05/31/2026 16:28:19.31
</commit_message>
<xml_diff>
--- a/WagonsWithWeight.xlsx
+++ b/WagonsWithWeight.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HAISB STORE\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8578473-0519-4183-A337-97FAE5671AE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD09B89B-E6EB-4F37-AB08-A82F654B5971}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8190" yWindow="1125" windowWidth="21600" windowHeight="11235" xr2:uid="{68AA4FA8-561F-47EB-AC86-75E02A3E7FE4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{68AA4FA8-561F-47EB-AC86-75E02A3E7FE4}"/>
   </bookViews>
   <sheets>
     <sheet name="WagonsWithWeight" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5138" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4646" uniqueCount="98">
   <si>
     <t>تاریخ</t>
   </si>
@@ -353,21 +353,6 @@
   <si>
     <t>چهار رنگه(نوری‌نان 45کیلو٬البرز٬فضا٬جهان)</t>
   </si>
-  <si>
-    <t>شاه</t>
-  </si>
-  <si>
-    <t>دورنگه(آتیلا نان ویش سورت٬ آتیلا نان ترمیده)</t>
-  </si>
-  <si>
-    <t>بچه چاپ سهاک</t>
-  </si>
-  <si>
-    <t>سه رنگه(بچه چاپ٬ منصور٬ رضوان)</t>
-  </si>
-  <si>
-    <t>پورت نمبر 5</t>
-  </si>
 </sst>
 </file>
 
@@ -590,6 +575,19 @@
         <top style="thin">
           <color indexed="64"/>
         </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
@@ -601,7 +599,9 @@
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
         <top style="thin">
           <color indexed="64"/>
         </top>
@@ -786,11 +786,10 @@
       </border>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="[$-16048C]yyyy/m/d;@"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
+        <left/>
         <right style="thin">
           <color indexed="64"/>
         </right>
@@ -817,31 +816,10 @@
       </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-16048C]yyyy/m/d;@"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
       <border>
         <top style="thin">
           <color indexed="64"/>
         </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -862,6 +840,13 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -927,6 +912,7 @@
       <sheetName val="Sheet1"/>
       <sheetName val="Sheet2"/>
       <sheetName val="Dashboard"/>
+      <sheetName val="MasterTableForAllWagons"/>
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
@@ -941,6 +927,7 @@
       <sheetData sheetId="9"/>
       <sheetData sheetId="10"/>
       <sheetData sheetId="11"/>
+      <sheetData sheetId="12" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1012,19 +999,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7A8B5CD-448E-48E3-8458-B8CC5030BD56}" name="Table6" displayName="Table6" ref="A1:H1711" headerRowDxfId="20" dataDxfId="19" headerRowBorderDxfId="17" tableBorderDxfId="18" totalsRowBorderDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7A8B5CD-448E-48E3-8458-B8CC5030BD56}" name="Table6" displayName="Table6" ref="A1:H1547" headerRowDxfId="20" dataDxfId="18" headerRowBorderDxfId="19" tableBorderDxfId="17" totalsRowBorderDxfId="16">
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H1340">
     <sortCondition ref="A1:A1340"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{FBB8F405-56D9-4C99-8154-1690E2919089}" name="تاریخ" totalsRowLabel="Total" dataDxfId="14" totalsRowDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{63A2DE36-8DEB-4848-BAD2-AA9F32B8B2DC}" name="اسم شرکت" dataDxfId="12" totalsRowDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{EE530A03-6AD4-4402-8DEA-FEC97A0CCA79}" name="نمبر واگون" totalsRowFunction="count" dataDxfId="10" totalsRowDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{9486619F-2E6A-4089-B90D-B4502A580386}" name="محل بارگیری" dataDxfId="8" totalsRowDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{0F903A3F-D4C2-4F15-82AB-7C7C61073477}" name="اسم ارد" dataDxfId="6" totalsRowDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{ECBC210B-9AE6-48CD-83D4-D214345D9E0C}" name="تعداد" dataDxfId="4" totalsRowDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{06846136-8155-46A1-A193-C22FFD89FD6C}" name="وزن" dataDxfId="2" totalsRowDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{2648665B-8FBB-47DC-B51F-E748C6255995}" name="تعدا کامیون" totalsRowFunction="sum" dataDxfId="0" totalsRowDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{FBB8F405-56D9-4C99-8154-1690E2919089}" name="تاریخ" totalsRowLabel="Total" dataDxfId="15" totalsRowDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{63A2DE36-8DEB-4848-BAD2-AA9F32B8B2DC}" name="اسم شرکت" dataDxfId="13" totalsRowDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{EE530A03-6AD4-4402-8DEA-FEC97A0CCA79}" name="نمبر واگون" totalsRowFunction="count" dataDxfId="11" totalsRowDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{9486619F-2E6A-4089-B90D-B4502A580386}" name="محل بارگیری" dataDxfId="9" totalsRowDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{0F903A3F-D4C2-4F15-82AB-7C7C61073477}" name="اسم ارد" dataDxfId="7" totalsRowDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{ECBC210B-9AE6-48CD-83D4-D214345D9E0C}" name="تعداد" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{06846136-8155-46A1-A193-C22FFD89FD6C}" name="وزن" dataDxfId="3" totalsRowDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{2648665B-8FBB-47DC-B51F-E748C6255995}" name="تعدا کامیون" totalsRowFunction="sum" dataDxfId="1" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1328,7 +1315,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26D80CA6-9C60-4A13-87BC-5BF4E6FD5B80}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:H1711"/>
+  <dimension ref="A1:H1547"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" style="11" bestFit="1" customWidth="1"/>
@@ -41563,4228 +41550,6 @@
         <v>3</v>
       </c>
     </row>
-    <row r="1548" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1548" s="5">
-        <v>46159</v>
-      </c>
-      <c r="B1548" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1548" s="6">
-        <v>28849677</v>
-      </c>
-      <c r="D1548" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1548" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1548" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1548" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1548" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1549" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1549" s="5">
-        <v>46159</v>
-      </c>
-      <c r="B1549" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1549" s="6">
-        <v>29096948</v>
-      </c>
-      <c r="D1549" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1549" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1549" s="6">
-        <v>1336</v>
-      </c>
-      <c r="G1549" s="6">
-        <v>66800</v>
-      </c>
-      <c r="H1549" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1550" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1550" s="5">
-        <v>46159</v>
-      </c>
-      <c r="B1550" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1550" s="6">
-        <v>28855559</v>
-      </c>
-      <c r="D1550" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1550" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1550" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1550" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1550" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1551" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1551" s="5">
-        <v>46159</v>
-      </c>
-      <c r="B1551" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1551" s="6">
-        <v>52629102</v>
-      </c>
-      <c r="D1551" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1551" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1551" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1551" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1551" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1552" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1552" s="5">
-        <v>46159</v>
-      </c>
-      <c r="B1552" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1552" s="6">
-        <v>29029956</v>
-      </c>
-      <c r="D1552" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1552" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1552" s="6">
-        <v>1340</v>
-      </c>
-      <c r="G1552" s="6">
-        <v>67000</v>
-      </c>
-      <c r="H1552" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1553" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1553" s="5">
-        <v>46159</v>
-      </c>
-      <c r="B1553" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1553" s="6">
-        <v>29140126</v>
-      </c>
-      <c r="D1553" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1553" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1553" s="6">
-        <v>1336</v>
-      </c>
-      <c r="G1553" s="6">
-        <v>66800</v>
-      </c>
-      <c r="H1553" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1554" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1554" s="5">
-        <v>46159</v>
-      </c>
-      <c r="B1554" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1554" s="6">
-        <v>29445301</v>
-      </c>
-      <c r="D1554" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1554" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1554" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1554" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1554" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1555" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1555" s="5">
-        <v>46159</v>
-      </c>
-      <c r="B1555" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1555" s="6">
-        <v>29140233</v>
-      </c>
-      <c r="D1555" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1555" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1555" s="6">
-        <v>1335</v>
-      </c>
-      <c r="G1555" s="6">
-        <v>66750</v>
-      </c>
-      <c r="H1555" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1556" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1556" s="5">
-        <v>46159</v>
-      </c>
-      <c r="B1556" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1556" s="6">
-        <v>28855948</v>
-      </c>
-      <c r="D1556" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1556" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1556" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1556" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1556" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1557" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1557" s="5">
-        <v>46159</v>
-      </c>
-      <c r="B1557" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1557" s="6">
-        <v>28853984</v>
-      </c>
-      <c r="D1557" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1557" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1557" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1557" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1557" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1558" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1558" s="5">
-        <v>46159</v>
-      </c>
-      <c r="B1558" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1558" s="6">
-        <v>28844926</v>
-      </c>
-      <c r="D1558" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1558" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1558" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1558" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1558" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1559" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1559" s="5">
-        <v>46159</v>
-      </c>
-      <c r="B1559" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1559" s="6">
-        <v>29300548</v>
-      </c>
-      <c r="D1559" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1559" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1559" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1559" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1559" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1560" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1560" s="5">
-        <v>46159</v>
-      </c>
-      <c r="B1560" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1560" s="6">
-        <v>29875499</v>
-      </c>
-      <c r="D1560" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1560" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1560" s="6">
-        <v>1340</v>
-      </c>
-      <c r="G1560" s="6">
-        <v>67000</v>
-      </c>
-      <c r="H1560" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1561" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1561" s="5">
-        <v>46159</v>
-      </c>
-      <c r="B1561" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1561" s="6">
-        <v>28849487</v>
-      </c>
-      <c r="D1561" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1561" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1561" s="6">
-        <v>1336</v>
-      </c>
-      <c r="G1561" s="6">
-        <v>66800</v>
-      </c>
-      <c r="H1561" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1562" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1562" s="5">
-        <v>46159</v>
-      </c>
-      <c r="B1562" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1562" s="6">
-        <v>28860369</v>
-      </c>
-      <c r="D1562" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1562" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="F1562" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1562" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1562" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1563" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1563" s="8">
-        <v>46159</v>
-      </c>
-      <c r="B1563" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1563" s="9">
-        <v>28841187</v>
-      </c>
-      <c r="D1563" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1563" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F1563" s="9">
-        <v>1356</v>
-      </c>
-      <c r="G1563" s="9">
-        <v>67800</v>
-      </c>
-      <c r="H1563" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1564" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1564" s="8">
-        <v>46159</v>
-      </c>
-      <c r="B1564" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1564" s="9">
-        <v>28021350</v>
-      </c>
-      <c r="D1564" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1564" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F1564" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1564" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1564" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1565" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1565" s="8">
-        <v>46159</v>
-      </c>
-      <c r="B1565" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1565" s="9">
-        <v>28046985</v>
-      </c>
-      <c r="D1565" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1565" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1565" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1565" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1565" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1566" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1566" s="8">
-        <v>46159</v>
-      </c>
-      <c r="B1566" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1566" s="9">
-        <v>28345064</v>
-      </c>
-      <c r="D1566" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1566" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1566" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1566" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1566" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1567" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1567" s="8">
-        <v>46159</v>
-      </c>
-      <c r="B1567" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1567" s="9">
-        <v>28808954</v>
-      </c>
-      <c r="D1567" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1567" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1567" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1567" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1567" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1568" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1568" s="8">
-        <v>46160</v>
-      </c>
-      <c r="B1568" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1568" s="9">
-        <v>29226081</v>
-      </c>
-      <c r="D1568" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1568" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1568" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1568" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1568" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1569" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1569" s="8">
-        <v>46160</v>
-      </c>
-      <c r="B1569" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1569" s="9">
-        <v>29841392</v>
-      </c>
-      <c r="D1569" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1569" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1569" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1569" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1569" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1570" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1570" s="8">
-        <v>46160</v>
-      </c>
-      <c r="B1570" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1570" s="9">
-        <v>29026465</v>
-      </c>
-      <c r="D1570" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1570" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1570" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1570" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1570" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1571" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1571" s="8">
-        <v>46160</v>
-      </c>
-      <c r="B1571" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1571" s="9">
-        <v>28841179</v>
-      </c>
-      <c r="D1571" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1571" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F1571" s="9">
-        <v>1356</v>
-      </c>
-      <c r="G1571" s="9">
-        <v>67800</v>
-      </c>
-      <c r="H1571" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1572" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1572" s="8">
-        <v>46160</v>
-      </c>
-      <c r="B1572" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1572" s="9">
-        <v>28027126</v>
-      </c>
-      <c r="D1572" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1572" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="F1572" s="9">
-        <v>1300</v>
-      </c>
-      <c r="G1572" s="9">
-        <v>65000</v>
-      </c>
-      <c r="H1572" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1573" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1573" s="8">
-        <v>46159</v>
-      </c>
-      <c r="B1573" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1573" s="9">
-        <v>98219330</v>
-      </c>
-      <c r="D1573" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1573" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="F1573" s="9">
-        <v>1246</v>
-      </c>
-      <c r="G1573" s="9">
-        <v>67600</v>
-      </c>
-      <c r="H1573" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1574" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1574" s="8">
-        <v>46159</v>
-      </c>
-      <c r="B1574" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1574" s="9">
-        <v>99618662</v>
-      </c>
-      <c r="D1574" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1574" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="F1574" s="9">
-        <v>1274</v>
-      </c>
-      <c r="G1574" s="9">
-        <v>67940</v>
-      </c>
-      <c r="H1574" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1575" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1575" s="8">
-        <v>46159</v>
-      </c>
-      <c r="B1575" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1575" s="9">
-        <v>95219010</v>
-      </c>
-      <c r="D1575" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1575" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="F1575" s="9">
-        <v>1256</v>
-      </c>
-      <c r="G1575" s="9">
-        <v>68210</v>
-      </c>
-      <c r="H1575" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1576" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1576" s="8">
-        <v>46159</v>
-      </c>
-      <c r="B1576" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1576" s="9">
-        <v>95276374</v>
-      </c>
-      <c r="D1576" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1576" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="F1576" s="9">
-        <v>1325</v>
-      </c>
-      <c r="G1576" s="9">
-        <v>67620</v>
-      </c>
-      <c r="H1576" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1577" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1577" s="8">
-        <v>46159</v>
-      </c>
-      <c r="B1577" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1577" s="9">
-        <v>98212657</v>
-      </c>
-      <c r="D1577" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1577" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="F1577" s="9">
-        <v>1258</v>
-      </c>
-      <c r="G1577" s="9">
-        <v>67700</v>
-      </c>
-      <c r="H1577" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1578" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1578" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1578" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1578" s="9">
-        <v>23562721</v>
-      </c>
-      <c r="D1578" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1578" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="F1578" s="9">
-        <v>1320</v>
-      </c>
-      <c r="G1578" s="9">
-        <v>66000</v>
-      </c>
-      <c r="H1578" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1579" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1579" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1579" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1579" s="9">
-        <v>23444763</v>
-      </c>
-      <c r="D1579" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1579" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="F1579" s="9">
-        <v>1320</v>
-      </c>
-      <c r="G1579" s="9">
-        <v>66000</v>
-      </c>
-      <c r="H1579" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1580" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1580" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1580" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1580" s="9">
-        <v>23568819</v>
-      </c>
-      <c r="D1580" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1580" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="F1580" s="9">
-        <v>1320</v>
-      </c>
-      <c r="G1580" s="9">
-        <v>66000</v>
-      </c>
-      <c r="H1580" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1581" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1581" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1581" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1581" s="9">
-        <v>87786190</v>
-      </c>
-      <c r="D1581" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1581" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="F1581" s="9">
-        <v>920</v>
-      </c>
-      <c r="G1581" s="9">
-        <v>46000</v>
-      </c>
-      <c r="H1581" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1582" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1582" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1582" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1582" s="9">
-        <v>87774592</v>
-      </c>
-      <c r="D1582" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1582" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="F1582" s="9">
-        <v>900</v>
-      </c>
-      <c r="G1582" s="9">
-        <v>45000</v>
-      </c>
-      <c r="H1582" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1583" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1583" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1583" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1583" s="9">
-        <v>91902163</v>
-      </c>
-      <c r="D1583" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1583" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="F1583" s="9">
-        <v>1000</v>
-      </c>
-      <c r="G1583" s="9">
-        <v>50000</v>
-      </c>
-      <c r="H1583" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1584" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1584" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1584" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1584" s="9">
-        <v>87787081</v>
-      </c>
-      <c r="D1584" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1584" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F1584" s="9">
-        <v>926</v>
-      </c>
-      <c r="G1584" s="9">
-        <v>46300</v>
-      </c>
-      <c r="H1584" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1585" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1585" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1585" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1585" s="9">
-        <v>87771689</v>
-      </c>
-      <c r="D1585" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1585" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F1585" s="9">
-        <v>900</v>
-      </c>
-      <c r="G1585" s="9">
-        <v>45000</v>
-      </c>
-      <c r="H1585" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1586" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1586" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1586" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1586" s="9">
-        <v>91916478</v>
-      </c>
-      <c r="D1586" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1586" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="F1586" s="9">
-        <v>1000</v>
-      </c>
-      <c r="G1586" s="9">
-        <v>50000</v>
-      </c>
-      <c r="H1586" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1587" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1587" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1587" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1587" s="9">
-        <v>29927894</v>
-      </c>
-      <c r="D1587" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1587" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1587" s="9">
-        <v>1340</v>
-      </c>
-      <c r="G1587" s="9">
-        <v>67000</v>
-      </c>
-      <c r="H1587" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1588" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1588" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1588" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1588" s="9">
-        <v>29441565</v>
-      </c>
-      <c r="D1588" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1588" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1588" s="9">
-        <v>1356</v>
-      </c>
-      <c r="G1588" s="9">
-        <v>67800</v>
-      </c>
-      <c r="H1588" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1589" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1589" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1589" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1589" s="9">
-        <v>28863371</v>
-      </c>
-      <c r="D1589" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1589" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1589" s="9">
-        <v>1356</v>
-      </c>
-      <c r="G1589" s="9">
-        <v>67800</v>
-      </c>
-      <c r="H1589" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1590" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1590" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1590" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1590" s="9">
-        <v>91914226</v>
-      </c>
-      <c r="D1590" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1590" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="F1590" s="9">
-        <v>998</v>
-      </c>
-      <c r="G1590" s="9">
-        <v>49900</v>
-      </c>
-      <c r="H1590" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1591" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1591" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1591" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1591" s="9">
-        <v>91914259</v>
-      </c>
-      <c r="D1591" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1591" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="F1591" s="9">
-        <v>1000</v>
-      </c>
-      <c r="G1591" s="9">
-        <v>50000</v>
-      </c>
-      <c r="H1591" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1592" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1592" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1592" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1592" s="9">
-        <v>91917427</v>
-      </c>
-      <c r="D1592" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1592" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="F1592" s="9">
-        <v>1000</v>
-      </c>
-      <c r="G1592" s="9">
-        <v>50000</v>
-      </c>
-      <c r="H1592" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1593" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1593" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1593" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1593" s="9">
-        <v>91914242</v>
-      </c>
-      <c r="D1593" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1593" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="F1593" s="9">
-        <v>1000</v>
-      </c>
-      <c r="G1593" s="9">
-        <v>50000</v>
-      </c>
-      <c r="H1593" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1594" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1594" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1594" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1594" s="9">
-        <v>28861086</v>
-      </c>
-      <c r="D1594" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1594" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F1594" s="9">
-        <v>1356</v>
-      </c>
-      <c r="G1594" s="9">
-        <v>67800</v>
-      </c>
-      <c r="H1594" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1595" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1595" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1595" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1595" s="9">
-        <v>28841781</v>
-      </c>
-      <c r="D1595" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1595" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F1595" s="9">
-        <v>1356</v>
-      </c>
-      <c r="G1595" s="9">
-        <v>67800</v>
-      </c>
-      <c r="H1595" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1596" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1596" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1596" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1596" s="9">
-        <v>28865186</v>
-      </c>
-      <c r="D1596" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1596" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F1596" s="9">
-        <v>1356</v>
-      </c>
-      <c r="G1596" s="9">
-        <v>67800</v>
-      </c>
-      <c r="H1596" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1597" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1597" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1597" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1597" s="9">
-        <v>28858975</v>
-      </c>
-      <c r="D1597" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1597" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F1597" s="9">
-        <v>1356</v>
-      </c>
-      <c r="G1597" s="9">
-        <v>67800</v>
-      </c>
-      <c r="H1597" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1598" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1598" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1598" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1598" s="9">
-        <v>28865178</v>
-      </c>
-      <c r="D1598" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1598" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F1598" s="9">
-        <v>1355</v>
-      </c>
-      <c r="G1598" s="9">
-        <v>67750</v>
-      </c>
-      <c r="H1598" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1599" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1599" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1599" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1599" s="9">
-        <v>28841500</v>
-      </c>
-      <c r="D1599" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1599" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F1599" s="9">
-        <v>1356</v>
-      </c>
-      <c r="G1599" s="9">
-        <v>67800</v>
-      </c>
-      <c r="H1599" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1600" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1600" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1600" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1600" s="9">
-        <v>28863975</v>
-      </c>
-      <c r="D1600" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1600" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F1600" s="9">
-        <v>1356</v>
-      </c>
-      <c r="G1600" s="9">
-        <v>67800</v>
-      </c>
-      <c r="H1600" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1601" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1601" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1601" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1601" s="9">
-        <v>28863660</v>
-      </c>
-      <c r="D1601" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1601" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F1601" s="9">
-        <v>1356</v>
-      </c>
-      <c r="G1601" s="9">
-        <v>67800</v>
-      </c>
-      <c r="H1601" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1602" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1602" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1602" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1602" s="9">
-        <v>28840403</v>
-      </c>
-      <c r="D1602" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1602" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F1602" s="9">
-        <v>1356</v>
-      </c>
-      <c r="G1602" s="9">
-        <v>67800</v>
-      </c>
-      <c r="H1602" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1603" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1603" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1603" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1603" s="9">
-        <v>28840379</v>
-      </c>
-      <c r="D1603" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1603" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F1603" s="9">
-        <v>1356</v>
-      </c>
-      <c r="G1603" s="9">
-        <v>67800</v>
-      </c>
-      <c r="H1603" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1604" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1604" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1604" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1604" s="9">
-        <v>28814572</v>
-      </c>
-      <c r="D1604" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1604" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1604" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1604" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1604" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1605" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1605" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1605" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1605" s="9">
-        <v>28345700</v>
-      </c>
-      <c r="D1605" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1605" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1605" s="9">
-        <v>1350</v>
-      </c>
-      <c r="G1605" s="9">
-        <v>67500</v>
-      </c>
-      <c r="H1605" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1606" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1606" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1606" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1606" s="9">
-        <v>28043487</v>
-      </c>
-      <c r="D1606" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1606" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1606" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1606" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1606" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1607" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1607" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1607" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1607" s="9">
-        <v>28801389</v>
-      </c>
-      <c r="D1607" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1607" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1607" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1607" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1607" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1608" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1608" s="8">
-        <v>46161</v>
-      </c>
-      <c r="B1608" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1608" s="9">
-        <v>28060267</v>
-      </c>
-      <c r="D1608" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1608" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="F1608" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1608" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1608" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1609" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1609" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1609" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1609" s="6">
-        <v>28040236</v>
-      </c>
-      <c r="D1609" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1609" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="F1609" s="6">
-        <v>1360</v>
-      </c>
-      <c r="G1609" s="6">
-        <v>68000</v>
-      </c>
-      <c r="H1609" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1610" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1610" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1610" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1610" s="6">
-        <v>29001401</v>
-      </c>
-      <c r="D1610" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1610" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="F1610" s="6">
-        <v>1360</v>
-      </c>
-      <c r="G1610" s="6">
-        <v>68000</v>
-      </c>
-      <c r="H1610" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1611" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1611" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1611" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1611" s="6">
-        <v>28077717</v>
-      </c>
-      <c r="D1611" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1611" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="F1611" s="6">
-        <v>1360</v>
-      </c>
-      <c r="G1611" s="6">
-        <v>68000</v>
-      </c>
-      <c r="H1611" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1612" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1612" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1612" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1612" s="6">
-        <v>29145489</v>
-      </c>
-      <c r="D1612" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1612" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="F1612" s="6">
-        <v>1300</v>
-      </c>
-      <c r="G1612" s="6">
-        <v>65000</v>
-      </c>
-      <c r="H1612" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1613" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1613" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1613" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1613" s="6">
-        <v>87817599</v>
-      </c>
-      <c r="D1613" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1613" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="F1613" s="6">
-        <v>980</v>
-      </c>
-      <c r="G1613" s="6">
-        <v>49000</v>
-      </c>
-      <c r="H1613" s="7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1614" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1614" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1614" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1614" s="6">
-        <v>91901645</v>
-      </c>
-      <c r="D1614" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1614" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="F1614" s="6">
-        <v>1000</v>
-      </c>
-      <c r="G1614" s="6">
-        <v>50000</v>
-      </c>
-      <c r="H1614" s="7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1615" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1615" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1615" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1615" s="6">
-        <v>87782181</v>
-      </c>
-      <c r="D1615" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1615" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="F1615" s="6">
-        <v>900</v>
-      </c>
-      <c r="G1615" s="6">
-        <v>45000</v>
-      </c>
-      <c r="H1615" s="7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1616" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1616" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1616" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1616" s="6">
-        <v>28873560</v>
-      </c>
-      <c r="D1616" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1616" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1616" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1616" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1616" s="7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1617" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1617" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1617" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1617" s="6">
-        <v>29026663</v>
-      </c>
-      <c r="D1617" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1617" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1617" s="6">
-        <v>1340</v>
-      </c>
-      <c r="G1617" s="6">
-        <v>67000</v>
-      </c>
-      <c r="H1617" s="7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1618" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1618" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1618" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1618" s="6">
-        <v>28865632</v>
-      </c>
-      <c r="D1618" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1618" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1618" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1618" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1618" s="7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1619" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1619" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1619" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1619" s="6">
-        <v>29222635</v>
-      </c>
-      <c r="D1619" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1619" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1619" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1619" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1619" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1620" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1620" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1620" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1620" s="6">
-        <v>29222627</v>
-      </c>
-      <c r="D1620" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1620" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1620" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1620" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1620" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1621" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1621" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1621" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1621" s="6">
-        <v>28840916</v>
-      </c>
-      <c r="D1621" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1621" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="F1621" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1621" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1621" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1622" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1622" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1622" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1622" s="6">
-        <v>28841401</v>
-      </c>
-      <c r="D1622" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1622" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="F1622" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1622" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1622" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1623" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1623" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1623" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1623" s="6">
-        <v>29305216</v>
-      </c>
-      <c r="D1623" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1623" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="F1623" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1623" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1623" s="7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1624" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1624" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1624" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1624" s="6">
-        <v>29452521</v>
-      </c>
-      <c r="D1624" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1624" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="F1624" s="6">
-        <v>1355</v>
-      </c>
-      <c r="G1624" s="6">
-        <v>67750</v>
-      </c>
-      <c r="H1624" s="7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1625" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1625" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1625" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1625" s="6">
-        <v>29452232</v>
-      </c>
-      <c r="D1625" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1625" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="F1625" s="6">
-        <v>1354</v>
-      </c>
-      <c r="G1625" s="6">
-        <v>67700</v>
-      </c>
-      <c r="H1625" s="7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1626" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1626" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1626" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1626" s="6">
-        <v>28044477</v>
-      </c>
-      <c r="D1626" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1626" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1626" s="6">
-        <v>1360</v>
-      </c>
-      <c r="G1626" s="6">
-        <v>68000</v>
-      </c>
-      <c r="H1626" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1627" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1627" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1627" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1627" s="6">
-        <v>28053445</v>
-      </c>
-      <c r="D1627" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1627" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1627" s="6">
-        <v>1360</v>
-      </c>
-      <c r="G1627" s="6">
-        <v>68000</v>
-      </c>
-      <c r="H1627" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1628" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1628" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1628" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1628" s="6">
-        <v>28814523</v>
-      </c>
-      <c r="D1628" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1628" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="F1628" s="6">
-        <v>1360</v>
-      </c>
-      <c r="G1628" s="6">
-        <v>68000</v>
-      </c>
-      <c r="H1628" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1629" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1629" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1629" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1629" s="6">
-        <v>28289395</v>
-      </c>
-      <c r="D1629" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1629" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="F1629" s="6">
-        <v>1340</v>
-      </c>
-      <c r="G1629" s="6">
-        <v>67000</v>
-      </c>
-      <c r="H1629" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1630" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1630" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1630" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1630" s="6">
-        <v>28015352</v>
-      </c>
-      <c r="D1630" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1630" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="F1630" s="6">
-        <v>1360</v>
-      </c>
-      <c r="G1630" s="6">
-        <v>68000</v>
-      </c>
-      <c r="H1630" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1631" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1631" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1631" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1631" s="6">
-        <v>28010403</v>
-      </c>
-      <c r="D1631" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1631" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="F1631" s="6">
-        <v>1360</v>
-      </c>
-      <c r="G1631" s="6">
-        <v>68000</v>
-      </c>
-      <c r="H1631" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1632" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1632" s="5">
-        <v>46162</v>
-      </c>
-      <c r="B1632" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1632" s="6">
-        <v>28010775</v>
-      </c>
-      <c r="D1632" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1632" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="F1632" s="6">
-        <v>1360</v>
-      </c>
-      <c r="G1632" s="6">
-        <v>68000</v>
-      </c>
-      <c r="H1632" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1633" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1633" s="8">
-        <v>46162</v>
-      </c>
-      <c r="B1633" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1633" s="9">
-        <v>28347201</v>
-      </c>
-      <c r="D1633" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1633" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="F1633" s="9">
-        <v>1257</v>
-      </c>
-      <c r="G1633" s="9">
-        <v>62850</v>
-      </c>
-      <c r="H1633" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1634" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1634" s="8">
-        <v>46162</v>
-      </c>
-      <c r="B1634" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1634" s="9">
-        <v>98215205</v>
-      </c>
-      <c r="D1634" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1634" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="F1634" s="9">
-        <v>1190</v>
-      </c>
-      <c r="G1634" s="9">
-        <v>68530</v>
-      </c>
-      <c r="H1634" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1635" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1635" s="8">
-        <v>46162</v>
-      </c>
-      <c r="B1635" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1635" s="9">
-        <v>98219306</v>
-      </c>
-      <c r="D1635" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1635" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="F1635" s="9">
-        <v>1170</v>
-      </c>
-      <c r="G1635" s="9">
-        <v>70360</v>
-      </c>
-      <c r="H1635" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1636" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1636" s="8">
-        <v>46162</v>
-      </c>
-      <c r="B1636" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1636" s="9">
-        <v>99409310</v>
-      </c>
-      <c r="D1636" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1636" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="F1636" s="9">
-        <v>1197</v>
-      </c>
-      <c r="G1636" s="9">
-        <v>68320</v>
-      </c>
-      <c r="H1636" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1637" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1637" s="8">
-        <v>46162</v>
-      </c>
-      <c r="B1637" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1637" s="9">
-        <v>28841153</v>
-      </c>
-      <c r="D1637" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1637" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F1637" s="9">
-        <v>1356</v>
-      </c>
-      <c r="G1637" s="9">
-        <v>67800</v>
-      </c>
-      <c r="H1637" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1638" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1638" s="8">
-        <v>46162</v>
-      </c>
-      <c r="B1638" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1638" s="9">
-        <v>28840437</v>
-      </c>
-      <c r="D1638" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1638" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F1638" s="9">
-        <v>1356</v>
-      </c>
-      <c r="G1638" s="9">
-        <v>67800</v>
-      </c>
-      <c r="H1638" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1639" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1639" s="8">
-        <v>46162</v>
-      </c>
-      <c r="B1639" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1639" s="9">
-        <v>28863512</v>
-      </c>
-      <c r="D1639" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1639" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1639" s="9">
-        <v>1356</v>
-      </c>
-      <c r="G1639" s="9">
-        <v>67800</v>
-      </c>
-      <c r="H1639" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1640" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1640" s="8">
-        <v>46162</v>
-      </c>
-      <c r="B1640" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1640" s="9">
-        <v>28090983</v>
-      </c>
-      <c r="D1640" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1640" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1640" s="9">
-        <v>1356</v>
-      </c>
-      <c r="G1640" s="9">
-        <v>67800</v>
-      </c>
-      <c r="H1640" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1641" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1641" s="8">
-        <v>46163</v>
-      </c>
-      <c r="B1641" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1641" s="9">
-        <v>91901637</v>
-      </c>
-      <c r="D1641" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1641" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="F1641" s="9">
-        <v>1000</v>
-      </c>
-      <c r="G1641" s="9">
-        <v>50000</v>
-      </c>
-      <c r="H1641" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1642" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1642" s="8">
-        <v>46163</v>
-      </c>
-      <c r="B1642" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1642" s="9">
-        <v>91901652</v>
-      </c>
-      <c r="D1642" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1642" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="F1642" s="9">
-        <v>1000</v>
-      </c>
-      <c r="G1642" s="9">
-        <v>50000</v>
-      </c>
-      <c r="H1642" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1643" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1643" s="8">
-        <v>46163</v>
-      </c>
-      <c r="B1643" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1643" s="9">
-        <v>91913160</v>
-      </c>
-      <c r="D1643" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1643" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="F1643" s="9">
-        <v>1000</v>
-      </c>
-      <c r="G1643" s="9">
-        <v>50000</v>
-      </c>
-      <c r="H1643" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1644" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1644" s="8">
-        <v>46163</v>
-      </c>
-      <c r="B1644" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1644" s="9">
-        <v>28040756</v>
-      </c>
-      <c r="D1644" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1644" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1644" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1644" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1644" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1645" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1645" s="8">
-        <v>46163</v>
-      </c>
-      <c r="B1645" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1645" s="9">
-        <v>28054153</v>
-      </c>
-      <c r="D1645" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1645" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1645" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1645" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1645" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1646" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1646" s="8">
-        <v>46163</v>
-      </c>
-      <c r="B1646" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1646" s="9">
-        <v>28820116</v>
-      </c>
-      <c r="D1646" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1646" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1646" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1646" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1646" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1647" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1647" s="8">
-        <v>46163</v>
-      </c>
-      <c r="B1647" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1647" s="9">
-        <v>28021756</v>
-      </c>
-      <c r="D1647" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1647" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F1647" s="9">
-        <v>1358</v>
-      </c>
-      <c r="G1647" s="9">
-        <v>67900</v>
-      </c>
-      <c r="H1647" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1648" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1648" s="8">
-        <v>46163</v>
-      </c>
-      <c r="B1648" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1648" s="9">
-        <v>28011559</v>
-      </c>
-      <c r="D1648" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1648" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1648" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1648" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1648" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1649" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1649" s="8">
-        <v>46163</v>
-      </c>
-      <c r="B1649" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1649" s="9">
-        <v>28821551</v>
-      </c>
-      <c r="D1649" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1649" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1649" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1649" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1649" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1650" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1650" s="8">
-        <v>46163</v>
-      </c>
-      <c r="B1650" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1650" s="9">
-        <v>28010569</v>
-      </c>
-      <c r="D1650" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1650" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1650" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1650" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1650" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1651" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1651" s="8">
-        <v>46163</v>
-      </c>
-      <c r="B1651" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1651" s="9">
-        <v>29109477</v>
-      </c>
-      <c r="D1651" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1651" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="F1651" s="9">
-        <v>1336</v>
-      </c>
-      <c r="G1651" s="9">
-        <v>66800</v>
-      </c>
-      <c r="H1651" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1652" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1652" s="8">
-        <v>46163</v>
-      </c>
-      <c r="B1652" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1652" s="9">
-        <v>29900198</v>
-      </c>
-      <c r="D1652" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1652" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="F1652" s="9">
-        <v>1339</v>
-      </c>
-      <c r="G1652" s="9">
-        <v>66950</v>
-      </c>
-      <c r="H1652" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1653" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1653" s="8">
-        <v>46163</v>
-      </c>
-      <c r="B1653" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1653" s="9">
-        <v>28345403</v>
-      </c>
-      <c r="D1653" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1653" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="F1653" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1653" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1653" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1654" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1654" s="8">
-        <v>46163</v>
-      </c>
-      <c r="B1654" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1654" s="9">
-        <v>28815173</v>
-      </c>
-      <c r="D1654" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1654" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="F1654" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1654" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1654" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1655" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1655" s="8">
-        <v>46164</v>
-      </c>
-      <c r="B1655" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1655" s="9">
-        <v>29140340</v>
-      </c>
-      <c r="D1655" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1655" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1655" s="9">
-        <v>1336</v>
-      </c>
-      <c r="G1655" s="9">
-        <v>66800</v>
-      </c>
-      <c r="H1655" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1656" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1656" s="8">
-        <v>46164</v>
-      </c>
-      <c r="B1656" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1656" s="9">
-        <v>28022754</v>
-      </c>
-      <c r="D1656" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1656" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F1656" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1656" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1656" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1657" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1657" s="8">
-        <v>46164</v>
-      </c>
-      <c r="B1657" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1657" s="9">
-        <v>28808046</v>
-      </c>
-      <c r="D1657" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1657" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1657" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1657" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1657" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1658" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1658" s="8">
-        <v>46164</v>
-      </c>
-      <c r="B1658" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1658" s="9">
-        <v>28051902</v>
-      </c>
-      <c r="D1658" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1658" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1658" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1658" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1658" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1659" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1659" s="8">
-        <v>46164</v>
-      </c>
-      <c r="B1659" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1659" s="9">
-        <v>28051621</v>
-      </c>
-      <c r="D1659" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1659" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1659" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1659" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1659" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1660" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1660" s="8">
-        <v>46164</v>
-      </c>
-      <c r="B1660" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1660" s="9">
-        <v>28023745</v>
-      </c>
-      <c r="D1660" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1660" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1660" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1660" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1660" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1661" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1661" s="8">
-        <v>46164</v>
-      </c>
-      <c r="B1661" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1661" s="9">
-        <v>28047389</v>
-      </c>
-      <c r="D1661" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1661" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="F1661" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1661" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1661" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1662" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1662" s="8">
-        <v>46164</v>
-      </c>
-      <c r="B1662" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1662" s="9">
-        <v>28346229</v>
-      </c>
-      <c r="D1662" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1662" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="F1662" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1662" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1662" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1663" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1663" s="8">
-        <v>46164</v>
-      </c>
-      <c r="B1663" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1663" s="9">
-        <v>28012318</v>
-      </c>
-      <c r="D1663" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1663" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="F1663" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1663" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1663" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1664" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1664" s="8">
-        <v>46164</v>
-      </c>
-      <c r="B1664" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1664" s="9">
-        <v>28045664</v>
-      </c>
-      <c r="D1664" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1664" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="F1664" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1664" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1664" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1665" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1665" s="8">
-        <v>46164</v>
-      </c>
-      <c r="B1665" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1665" s="9">
-        <v>28045151</v>
-      </c>
-      <c r="D1665" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1665" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="F1665" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1665" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1665" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1666" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1666" s="8">
-        <v>46164</v>
-      </c>
-      <c r="B1666" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1666" s="9">
-        <v>24671455</v>
-      </c>
-      <c r="D1666" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1666" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="F1666" s="9">
-        <v>1210</v>
-      </c>
-      <c r="G1666" s="9">
-        <v>60500</v>
-      </c>
-      <c r="H1666" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1667" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1667" s="8">
-        <v>46164</v>
-      </c>
-      <c r="B1667" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1667" s="9">
-        <v>28348522</v>
-      </c>
-      <c r="D1667" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1667" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="F1667" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1667" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1667" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1668" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1668" s="8">
-        <v>46164</v>
-      </c>
-      <c r="B1668" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1668" s="9">
-        <v>28801306</v>
-      </c>
-      <c r="D1668" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1668" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="F1668" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1668" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1668" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1669" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1669" s="8">
-        <v>46164</v>
-      </c>
-      <c r="B1669" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1669" s="9">
-        <v>28025344</v>
-      </c>
-      <c r="D1669" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="E1669" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="F1669" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1669" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1669" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1670" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1670" s="8">
-        <v>46164</v>
-      </c>
-      <c r="B1670" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1670" s="9">
-        <v>28059061</v>
-      </c>
-      <c r="D1670" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="E1670" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="F1670" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1670" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1670" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1671" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1671" s="8">
-        <v>46164</v>
-      </c>
-      <c r="B1671" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1671" s="9">
-        <v>28818904</v>
-      </c>
-      <c r="D1671" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="E1671" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="F1671" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1671" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1671" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1672" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1672" s="8">
-        <v>46164</v>
-      </c>
-      <c r="B1672" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1672" s="9">
-        <v>28801546</v>
-      </c>
-      <c r="D1672" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="E1672" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="F1672" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1672" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1672" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1673" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1673" s="8">
-        <v>46165</v>
-      </c>
-      <c r="B1673" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1673" s="9">
-        <v>28887750</v>
-      </c>
-      <c r="D1673" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1673" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="F1673" s="9">
-        <v>1356</v>
-      </c>
-      <c r="G1673" s="9">
-        <v>67800</v>
-      </c>
-      <c r="H1673" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1674" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1674" s="8">
-        <v>46165</v>
-      </c>
-      <c r="B1674" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1674" s="9">
-        <v>29445285</v>
-      </c>
-      <c r="D1674" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1674" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1674" s="9">
-        <v>1356</v>
-      </c>
-      <c r="G1674" s="9">
-        <v>67800</v>
-      </c>
-      <c r="H1674" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1675" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1675" s="8">
-        <v>46165</v>
-      </c>
-      <c r="B1675" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1675" s="9">
-        <v>29238540</v>
-      </c>
-      <c r="D1675" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1675" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1675" s="9">
-        <v>1356</v>
-      </c>
-      <c r="G1675" s="9">
-        <v>67800</v>
-      </c>
-      <c r="H1675" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1676" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1676" s="8">
-        <v>46165</v>
-      </c>
-      <c r="B1676" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1676" s="9">
-        <v>28351336</v>
-      </c>
-      <c r="D1676" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1676" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F1676" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1676" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1676" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1677" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1677" s="8">
-        <v>46165</v>
-      </c>
-      <c r="B1677" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1677" s="9">
-        <v>23539950</v>
-      </c>
-      <c r="D1677" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1677" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F1677" s="9">
-        <v>1320</v>
-      </c>
-      <c r="G1677" s="9">
-        <v>66000</v>
-      </c>
-      <c r="H1677" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1678" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1678" s="8">
-        <v>46165</v>
-      </c>
-      <c r="B1678" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1678" s="9">
-        <v>24343063</v>
-      </c>
-      <c r="D1678" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1678" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F1678" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1678" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1678" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1679" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1679" s="8">
-        <v>46165</v>
-      </c>
-      <c r="B1679" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1679" s="9">
-        <v>26230490</v>
-      </c>
-      <c r="D1679" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1679" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F1679" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1679" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1679" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1680" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1680" s="8">
-        <v>46165</v>
-      </c>
-      <c r="B1680" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1680" s="9">
-        <v>24425761</v>
-      </c>
-      <c r="D1680" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1680" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F1680" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1680" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1680" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1681" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1681" s="8">
-        <v>46165</v>
-      </c>
-      <c r="B1681" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1681" s="9">
-        <v>91916502</v>
-      </c>
-      <c r="D1681" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1681" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="F1681" s="9">
-        <v>1000</v>
-      </c>
-      <c r="G1681" s="9">
-        <v>50000</v>
-      </c>
-      <c r="H1681" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1682" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1682" s="8">
-        <v>46165</v>
-      </c>
-      <c r="B1682" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1682" s="9">
-        <v>87782157</v>
-      </c>
-      <c r="D1682" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1682" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="F1682" s="9">
-        <v>900</v>
-      </c>
-      <c r="G1682" s="9">
-        <v>45000</v>
-      </c>
-      <c r="H1682" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1683" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1683" s="8">
-        <v>46165</v>
-      </c>
-      <c r="B1683" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1683" s="9">
-        <v>87795795</v>
-      </c>
-      <c r="D1683" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1683" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="F1683" s="9">
-        <v>900</v>
-      </c>
-      <c r="G1683" s="9">
-        <v>45000</v>
-      </c>
-      <c r="H1683" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1684" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1684" s="8">
-        <v>46165</v>
-      </c>
-      <c r="B1684" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1684" s="9">
-        <v>91916486</v>
-      </c>
-      <c r="D1684" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1684" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="F1684" s="9">
-        <v>920</v>
-      </c>
-      <c r="G1684" s="9">
-        <v>46000</v>
-      </c>
-      <c r="H1684" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1685" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1685" s="8">
-        <v>46165</v>
-      </c>
-      <c r="B1685" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1685" s="9">
-        <v>23546906</v>
-      </c>
-      <c r="D1685" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1685" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="F1685" s="9">
-        <v>1280</v>
-      </c>
-      <c r="G1685" s="9">
-        <v>64000</v>
-      </c>
-      <c r="H1685" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1686" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1686" s="8">
-        <v>46165</v>
-      </c>
-      <c r="B1686" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1686" s="9">
-        <v>23470958</v>
-      </c>
-      <c r="D1686" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1686" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="F1686" s="9">
-        <v>1280</v>
-      </c>
-      <c r="G1686" s="9">
-        <v>64000</v>
-      </c>
-      <c r="H1686" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1687" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1687" s="8">
-        <v>46165</v>
-      </c>
-      <c r="B1687" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1687" s="9">
-        <v>28029346</v>
-      </c>
-      <c r="D1687" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1687" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F1687" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1687" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1687" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1688" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1688" s="8">
-        <v>46165</v>
-      </c>
-      <c r="B1688" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1688" s="9">
-        <v>24425852</v>
-      </c>
-      <c r="D1688" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1688" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F1688" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1688" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1688" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1689" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1689" s="8">
-        <v>46165</v>
-      </c>
-      <c r="B1689" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1689" s="9">
-        <v>28066751</v>
-      </c>
-      <c r="D1689" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1689" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F1689" s="9">
-        <v>1300</v>
-      </c>
-      <c r="G1689" s="9">
-        <v>65000</v>
-      </c>
-      <c r="H1689" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1690" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1690" s="8">
-        <v>46165</v>
-      </c>
-      <c r="B1690" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1690" s="9">
-        <v>52460466</v>
-      </c>
-      <c r="D1690" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1690" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F1690" s="9">
-        <v>1360</v>
-      </c>
-      <c r="G1690" s="9">
-        <v>68000</v>
-      </c>
-      <c r="H1690" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1691" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1691" s="5">
-        <v>46165</v>
-      </c>
-      <c r="B1691" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1691" s="6">
-        <v>28848133</v>
-      </c>
-      <c r="D1691" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1691" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F1691" s="6">
-        <v>1359</v>
-      </c>
-      <c r="G1691" s="6">
-        <v>67950</v>
-      </c>
-      <c r="H1691" s="7"/>
-    </row>
-    <row r="1692" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1692" s="5">
-        <v>46165</v>
-      </c>
-      <c r="B1692" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1692" s="6">
-        <v>28090264</v>
-      </c>
-      <c r="D1692" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1692" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F1692" s="6">
-        <v>1360</v>
-      </c>
-      <c r="G1692" s="6">
-        <v>68000</v>
-      </c>
-      <c r="H1692" s="7"/>
-    </row>
-    <row r="1693" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1693" s="5">
-        <v>46165</v>
-      </c>
-      <c r="B1693" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1693" s="6">
-        <v>28090785</v>
-      </c>
-      <c r="D1693" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1693" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F1693" s="6">
-        <v>1360</v>
-      </c>
-      <c r="G1693" s="6">
-        <v>68000</v>
-      </c>
-      <c r="H1693" s="7"/>
-    </row>
-    <row r="1694" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1694" s="5">
-        <v>46165</v>
-      </c>
-      <c r="B1694" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1694" s="6">
-        <v>28847770</v>
-      </c>
-      <c r="D1694" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1694" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F1694" s="6">
-        <v>1360</v>
-      </c>
-      <c r="G1694" s="6">
-        <v>68000</v>
-      </c>
-      <c r="H1694" s="7"/>
-    </row>
-    <row r="1695" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1695" s="5">
-        <v>46165</v>
-      </c>
-      <c r="B1695" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1695" s="6">
-        <v>28846830</v>
-      </c>
-      <c r="D1695" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1695" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F1695" s="6">
-        <v>1360</v>
-      </c>
-      <c r="G1695" s="6">
-        <v>68000</v>
-      </c>
-      <c r="H1695" s="7"/>
-    </row>
-    <row r="1696" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1696" s="5">
-        <v>46166</v>
-      </c>
-      <c r="B1696" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1696" s="6">
-        <v>29021144</v>
-      </c>
-      <c r="D1696" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1696" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1696" s="6">
-        <v>1360</v>
-      </c>
-      <c r="G1696" s="6">
-        <v>68000</v>
-      </c>
-      <c r="H1696" s="7"/>
-    </row>
-    <row r="1697" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1697" s="5">
-        <v>46166</v>
-      </c>
-      <c r="B1697" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1697" s="6">
-        <v>28002517</v>
-      </c>
-      <c r="D1697" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1697" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="F1697" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1697" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1697" s="7"/>
-    </row>
-    <row r="1698" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1698" s="5">
-        <v>46166</v>
-      </c>
-      <c r="B1698" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1698" s="6">
-        <v>29840592</v>
-      </c>
-      <c r="D1698" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1698" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="F1698" s="6">
-        <v>1340</v>
-      </c>
-      <c r="G1698" s="6">
-        <v>67000</v>
-      </c>
-      <c r="H1698" s="7"/>
-    </row>
-    <row r="1699" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1699" s="5">
-        <v>46166</v>
-      </c>
-      <c r="B1699" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1699" s="6">
-        <v>28855153</v>
-      </c>
-      <c r="D1699" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1699" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="F1699" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1699" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1699" s="7"/>
-    </row>
-    <row r="1700" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1700" s="5">
-        <v>46166</v>
-      </c>
-      <c r="B1700" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1700" s="6">
-        <v>28856086</v>
-      </c>
-      <c r="D1700" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1700" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="F1700" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1700" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1700" s="7"/>
-    </row>
-    <row r="1701" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1701" s="5">
-        <v>46166</v>
-      </c>
-      <c r="B1701" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1701" s="6">
-        <v>28854131</v>
-      </c>
-      <c r="D1701" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1701" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="F1701" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1701" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1701" s="7"/>
-    </row>
-    <row r="1702" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1702" s="5">
-        <v>46166</v>
-      </c>
-      <c r="B1702" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1702" s="6">
-        <v>28856144</v>
-      </c>
-      <c r="D1702" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1702" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="F1702" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1702" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1702" s="7"/>
-    </row>
-    <row r="1703" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1703" s="5">
-        <v>46166</v>
-      </c>
-      <c r="B1703" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1703" s="6">
-        <v>28856029</v>
-      </c>
-      <c r="D1703" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1703" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="F1703" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1703" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1703" s="7"/>
-    </row>
-    <row r="1704" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1704" s="5">
-        <v>46167</v>
-      </c>
-      <c r="B1704" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1704" s="6">
-        <v>29221074</v>
-      </c>
-      <c r="D1704" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1704" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1704" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1704" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1704" s="7"/>
-    </row>
-    <row r="1705" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1705" s="5">
-        <v>46167</v>
-      </c>
-      <c r="B1705" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1705" s="6">
-        <v>29410305</v>
-      </c>
-      <c r="D1705" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1705" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1705" s="6">
-        <v>1360</v>
-      </c>
-      <c r="G1705" s="6">
-        <v>68000</v>
-      </c>
-      <c r="H1705" s="7"/>
-    </row>
-    <row r="1706" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1706" s="5">
-        <v>46167</v>
-      </c>
-      <c r="B1706" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1706" s="6">
-        <v>29135431</v>
-      </c>
-      <c r="D1706" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1706" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1706" s="6">
-        <v>1360</v>
-      </c>
-      <c r="G1706" s="6">
-        <v>68000</v>
-      </c>
-      <c r="H1706" s="7"/>
-    </row>
-    <row r="1707" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1707" s="5">
-        <v>46167</v>
-      </c>
-      <c r="B1707" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1707" s="6">
-        <v>29221009</v>
-      </c>
-      <c r="D1707" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1707" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1707" s="6">
-        <v>1356</v>
-      </c>
-      <c r="G1707" s="6">
-        <v>67800</v>
-      </c>
-      <c r="H1707" s="7"/>
-    </row>
-    <row r="1708" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1708" s="5">
-        <v>46167</v>
-      </c>
-      <c r="B1708" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1708" s="6">
-        <v>28819480</v>
-      </c>
-      <c r="D1708" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1708" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1708" s="6">
-        <v>1360</v>
-      </c>
-      <c r="G1708" s="6">
-        <v>68000</v>
-      </c>
-      <c r="H1708" s="7"/>
-    </row>
-    <row r="1709" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1709" s="5">
-        <v>46167</v>
-      </c>
-      <c r="B1709" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1709" s="6">
-        <v>28349660</v>
-      </c>
-      <c r="D1709" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1709" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1709" s="6">
-        <v>1360</v>
-      </c>
-      <c r="G1709" s="6">
-        <v>68000</v>
-      </c>
-      <c r="H1709" s="7"/>
-    </row>
-    <row r="1710" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1710" s="5">
-        <v>46167</v>
-      </c>
-      <c r="B1710" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1710" s="6">
-        <v>28026961</v>
-      </c>
-      <c r="D1710" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1710" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1710" s="6">
-        <v>1360</v>
-      </c>
-      <c r="G1710" s="6">
-        <v>68000</v>
-      </c>
-      <c r="H1710" s="7"/>
-    </row>
-    <row r="1711" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1711" s="8">
-        <v>46166</v>
-      </c>
-      <c r="B1711" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1711" s="9">
-        <v>91138644</v>
-      </c>
-      <c r="D1711" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1711" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="F1711" s="9">
-        <v>1303</v>
-      </c>
-      <c r="G1711" s="9">
-        <v>68100</v>
-      </c>
-      <c r="H1711" s="10"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
auto update Sun 05/31/2026 17:08:53.40
</commit_message>
<xml_diff>
--- a/WagonsWithWeight.xlsx
+++ b/WagonsWithWeight.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HAISB STORE\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HAISB STORE\LME-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD09B89B-E6EB-4F37-AB08-A82F654B5971}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EBC20B8-DA38-47F4-ABFD-13EDF704A1F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{68AA4FA8-561F-47EB-AC86-75E02A3E7FE4}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4646" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5138" uniqueCount="103">
   <si>
     <t>تاریخ</t>
   </si>
@@ -352,6 +352,21 @@
   </si>
   <si>
     <t>چهار رنگه(نوری‌نان 45کیلو٬البرز٬فضا٬جهان)</t>
+  </si>
+  <si>
+    <t>شاه</t>
+  </si>
+  <si>
+    <t>دورنگه(آتیلا نان ویش سورت٬ آتیلا نان ترمیده)</t>
+  </si>
+  <si>
+    <t>بچه چاپ سهاک</t>
+  </si>
+  <si>
+    <t>سه رنگه(بچه چاپ٬ منصور٬ رضوان)</t>
+  </si>
+  <si>
+    <t>پورت نمبر 5</t>
   </si>
 </sst>
 </file>
@@ -1315,7 +1330,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26D80CA6-9C60-4A13-87BC-5BF4E6FD5B80}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:H1547"/>
+  <dimension ref="A1:H1711"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" style="11" bestFit="1" customWidth="1"/>
@@ -41550,6 +41565,4228 @@
         <v>3</v>
       </c>
     </row>
+    <row r="1548" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1548" s="5">
+        <v>46159</v>
+      </c>
+      <c r="B1548" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1548" s="6">
+        <v>28849677</v>
+      </c>
+      <c r="D1548" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1548" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1548" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1548" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1548" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1549" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1549" s="5">
+        <v>46159</v>
+      </c>
+      <c r="B1549" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1549" s="6">
+        <v>29096948</v>
+      </c>
+      <c r="D1549" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1549" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1549" s="6">
+        <v>1336</v>
+      </c>
+      <c r="G1549" s="6">
+        <v>66800</v>
+      </c>
+      <c r="H1549" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1550" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1550" s="5">
+        <v>46159</v>
+      </c>
+      <c r="B1550" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1550" s="6">
+        <v>28855559</v>
+      </c>
+      <c r="D1550" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1550" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1550" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1550" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1550" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1551" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1551" s="5">
+        <v>46159</v>
+      </c>
+      <c r="B1551" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1551" s="6">
+        <v>52629102</v>
+      </c>
+      <c r="D1551" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1551" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1551" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1551" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1551" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1552" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1552" s="5">
+        <v>46159</v>
+      </c>
+      <c r="B1552" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1552" s="6">
+        <v>29029956</v>
+      </c>
+      <c r="D1552" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1552" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1552" s="6">
+        <v>1340</v>
+      </c>
+      <c r="G1552" s="6">
+        <v>67000</v>
+      </c>
+      <c r="H1552" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1553" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1553" s="5">
+        <v>46159</v>
+      </c>
+      <c r="B1553" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1553" s="6">
+        <v>29140126</v>
+      </c>
+      <c r="D1553" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1553" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1553" s="6">
+        <v>1336</v>
+      </c>
+      <c r="G1553" s="6">
+        <v>66800</v>
+      </c>
+      <c r="H1553" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1554" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1554" s="5">
+        <v>46159</v>
+      </c>
+      <c r="B1554" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1554" s="6">
+        <v>29445301</v>
+      </c>
+      <c r="D1554" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1554" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1554" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1554" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1554" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1555" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1555" s="5">
+        <v>46159</v>
+      </c>
+      <c r="B1555" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1555" s="6">
+        <v>29140233</v>
+      </c>
+      <c r="D1555" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1555" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1555" s="6">
+        <v>1335</v>
+      </c>
+      <c r="G1555" s="6">
+        <v>66750</v>
+      </c>
+      <c r="H1555" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1556" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1556" s="5">
+        <v>46159</v>
+      </c>
+      <c r="B1556" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1556" s="6">
+        <v>28855948</v>
+      </c>
+      <c r="D1556" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1556" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1556" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1556" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1556" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1557" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1557" s="5">
+        <v>46159</v>
+      </c>
+      <c r="B1557" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1557" s="6">
+        <v>28853984</v>
+      </c>
+      <c r="D1557" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1557" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1557" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1557" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1557" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1558" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1558" s="5">
+        <v>46159</v>
+      </c>
+      <c r="B1558" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1558" s="6">
+        <v>28844926</v>
+      </c>
+      <c r="D1558" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1558" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1558" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1558" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1558" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1559" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1559" s="5">
+        <v>46159</v>
+      </c>
+      <c r="B1559" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1559" s="6">
+        <v>29300548</v>
+      </c>
+      <c r="D1559" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1559" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1559" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1559" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1559" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1560" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1560" s="5">
+        <v>46159</v>
+      </c>
+      <c r="B1560" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1560" s="6">
+        <v>29875499</v>
+      </c>
+      <c r="D1560" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1560" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1560" s="6">
+        <v>1340</v>
+      </c>
+      <c r="G1560" s="6">
+        <v>67000</v>
+      </c>
+      <c r="H1560" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1561" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1561" s="5">
+        <v>46159</v>
+      </c>
+      <c r="B1561" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1561" s="6">
+        <v>28849487</v>
+      </c>
+      <c r="D1561" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1561" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1561" s="6">
+        <v>1336</v>
+      </c>
+      <c r="G1561" s="6">
+        <v>66800</v>
+      </c>
+      <c r="H1561" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1562" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1562" s="5">
+        <v>46159</v>
+      </c>
+      <c r="B1562" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1562" s="6">
+        <v>28860369</v>
+      </c>
+      <c r="D1562" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1562" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1562" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1562" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1562" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1563" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1563" s="8">
+        <v>46159</v>
+      </c>
+      <c r="B1563" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1563" s="9">
+        <v>28841187</v>
+      </c>
+      <c r="D1563" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1563" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1563" s="9">
+        <v>1356</v>
+      </c>
+      <c r="G1563" s="9">
+        <v>67800</v>
+      </c>
+      <c r="H1563" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1564" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1564" s="8">
+        <v>46159</v>
+      </c>
+      <c r="B1564" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1564" s="9">
+        <v>28021350</v>
+      </c>
+      <c r="D1564" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1564" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1564" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1564" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1564" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1565" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1565" s="8">
+        <v>46159</v>
+      </c>
+      <c r="B1565" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1565" s="9">
+        <v>28046985</v>
+      </c>
+      <c r="D1565" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1565" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1565" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1565" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1565" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1566" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1566" s="8">
+        <v>46159</v>
+      </c>
+      <c r="B1566" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1566" s="9">
+        <v>28345064</v>
+      </c>
+      <c r="D1566" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1566" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1566" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1566" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1566" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1567" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1567" s="8">
+        <v>46159</v>
+      </c>
+      <c r="B1567" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1567" s="9">
+        <v>28808954</v>
+      </c>
+      <c r="D1567" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1567" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1567" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1567" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1567" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1568" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1568" s="8">
+        <v>46160</v>
+      </c>
+      <c r="B1568" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1568" s="9">
+        <v>29226081</v>
+      </c>
+      <c r="D1568" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1568" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1568" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1568" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1568" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1569" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1569" s="8">
+        <v>46160</v>
+      </c>
+      <c r="B1569" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1569" s="9">
+        <v>29841392</v>
+      </c>
+      <c r="D1569" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1569" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1569" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1569" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1569" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1570" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1570" s="8">
+        <v>46160</v>
+      </c>
+      <c r="B1570" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1570" s="9">
+        <v>29026465</v>
+      </c>
+      <c r="D1570" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1570" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1570" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1570" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1570" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1571" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1571" s="8">
+        <v>46160</v>
+      </c>
+      <c r="B1571" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1571" s="9">
+        <v>28841179</v>
+      </c>
+      <c r="D1571" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1571" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1571" s="9">
+        <v>1356</v>
+      </c>
+      <c r="G1571" s="9">
+        <v>67800</v>
+      </c>
+      <c r="H1571" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1572" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1572" s="8">
+        <v>46160</v>
+      </c>
+      <c r="B1572" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1572" s="9">
+        <v>28027126</v>
+      </c>
+      <c r="D1572" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1572" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1572" s="9">
+        <v>1300</v>
+      </c>
+      <c r="G1572" s="9">
+        <v>65000</v>
+      </c>
+      <c r="H1572" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1573" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1573" s="8">
+        <v>46159</v>
+      </c>
+      <c r="B1573" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1573" s="9">
+        <v>98219330</v>
+      </c>
+      <c r="D1573" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1573" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F1573" s="9">
+        <v>1246</v>
+      </c>
+      <c r="G1573" s="9">
+        <v>67600</v>
+      </c>
+      <c r="H1573" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1574" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1574" s="8">
+        <v>46159</v>
+      </c>
+      <c r="B1574" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1574" s="9">
+        <v>99618662</v>
+      </c>
+      <c r="D1574" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1574" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F1574" s="9">
+        <v>1274</v>
+      </c>
+      <c r="G1574" s="9">
+        <v>67940</v>
+      </c>
+      <c r="H1574" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1575" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1575" s="8">
+        <v>46159</v>
+      </c>
+      <c r="B1575" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1575" s="9">
+        <v>95219010</v>
+      </c>
+      <c r="D1575" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1575" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F1575" s="9">
+        <v>1256</v>
+      </c>
+      <c r="G1575" s="9">
+        <v>68210</v>
+      </c>
+      <c r="H1575" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1576" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1576" s="8">
+        <v>46159</v>
+      </c>
+      <c r="B1576" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1576" s="9">
+        <v>95276374</v>
+      </c>
+      <c r="D1576" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1576" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F1576" s="9">
+        <v>1325</v>
+      </c>
+      <c r="G1576" s="9">
+        <v>67620</v>
+      </c>
+      <c r="H1576" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1577" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1577" s="8">
+        <v>46159</v>
+      </c>
+      <c r="B1577" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1577" s="9">
+        <v>98212657</v>
+      </c>
+      <c r="D1577" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1577" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F1577" s="9">
+        <v>1258</v>
+      </c>
+      <c r="G1577" s="9">
+        <v>67700</v>
+      </c>
+      <c r="H1577" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1578" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1578" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1578" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1578" s="9">
+        <v>23562721</v>
+      </c>
+      <c r="D1578" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1578" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1578" s="9">
+        <v>1320</v>
+      </c>
+      <c r="G1578" s="9">
+        <v>66000</v>
+      </c>
+      <c r="H1578" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1579" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1579" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1579" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1579" s="9">
+        <v>23444763</v>
+      </c>
+      <c r="D1579" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1579" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="F1579" s="9">
+        <v>1320</v>
+      </c>
+      <c r="G1579" s="9">
+        <v>66000</v>
+      </c>
+      <c r="H1579" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1580" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1580" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1580" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1580" s="9">
+        <v>23568819</v>
+      </c>
+      <c r="D1580" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1580" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="F1580" s="9">
+        <v>1320</v>
+      </c>
+      <c r="G1580" s="9">
+        <v>66000</v>
+      </c>
+      <c r="H1580" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1581" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1581" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1581" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1581" s="9">
+        <v>87786190</v>
+      </c>
+      <c r="D1581" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1581" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="F1581" s="9">
+        <v>920</v>
+      </c>
+      <c r="G1581" s="9">
+        <v>46000</v>
+      </c>
+      <c r="H1581" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1582" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1582" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1582" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1582" s="9">
+        <v>87774592</v>
+      </c>
+      <c r="D1582" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1582" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="F1582" s="9">
+        <v>900</v>
+      </c>
+      <c r="G1582" s="9">
+        <v>45000</v>
+      </c>
+      <c r="H1582" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1583" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1583" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1583" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1583" s="9">
+        <v>91902163</v>
+      </c>
+      <c r="D1583" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1583" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="F1583" s="9">
+        <v>1000</v>
+      </c>
+      <c r="G1583" s="9">
+        <v>50000</v>
+      </c>
+      <c r="H1583" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1584" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1584" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1584" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1584" s="9">
+        <v>87787081</v>
+      </c>
+      <c r="D1584" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1584" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1584" s="9">
+        <v>926</v>
+      </c>
+      <c r="G1584" s="9">
+        <v>46300</v>
+      </c>
+      <c r="H1584" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1585" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1585" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1585" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1585" s="9">
+        <v>87771689</v>
+      </c>
+      <c r="D1585" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1585" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1585" s="9">
+        <v>900</v>
+      </c>
+      <c r="G1585" s="9">
+        <v>45000</v>
+      </c>
+      <c r="H1585" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1586" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1586" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1586" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1586" s="9">
+        <v>91916478</v>
+      </c>
+      <c r="D1586" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1586" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1586" s="9">
+        <v>1000</v>
+      </c>
+      <c r="G1586" s="9">
+        <v>50000</v>
+      </c>
+      <c r="H1586" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1587" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1587" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1587" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1587" s="9">
+        <v>29927894</v>
+      </c>
+      <c r="D1587" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1587" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1587" s="9">
+        <v>1340</v>
+      </c>
+      <c r="G1587" s="9">
+        <v>67000</v>
+      </c>
+      <c r="H1587" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1588" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1588" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1588" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1588" s="9">
+        <v>29441565</v>
+      </c>
+      <c r="D1588" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1588" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1588" s="9">
+        <v>1356</v>
+      </c>
+      <c r="G1588" s="9">
+        <v>67800</v>
+      </c>
+      <c r="H1588" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1589" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1589" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1589" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1589" s="9">
+        <v>28863371</v>
+      </c>
+      <c r="D1589" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1589" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1589" s="9">
+        <v>1356</v>
+      </c>
+      <c r="G1589" s="9">
+        <v>67800</v>
+      </c>
+      <c r="H1589" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1590" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1590" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1590" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1590" s="9">
+        <v>91914226</v>
+      </c>
+      <c r="D1590" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1590" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="F1590" s="9">
+        <v>998</v>
+      </c>
+      <c r="G1590" s="9">
+        <v>49900</v>
+      </c>
+      <c r="H1590" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1591" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1591" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1591" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1591" s="9">
+        <v>91914259</v>
+      </c>
+      <c r="D1591" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1591" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="F1591" s="9">
+        <v>1000</v>
+      </c>
+      <c r="G1591" s="9">
+        <v>50000</v>
+      </c>
+      <c r="H1591" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1592" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1592" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1592" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1592" s="9">
+        <v>91917427</v>
+      </c>
+      <c r="D1592" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1592" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="F1592" s="9">
+        <v>1000</v>
+      </c>
+      <c r="G1592" s="9">
+        <v>50000</v>
+      </c>
+      <c r="H1592" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1593" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1593" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1593" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1593" s="9">
+        <v>91914242</v>
+      </c>
+      <c r="D1593" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1593" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="F1593" s="9">
+        <v>1000</v>
+      </c>
+      <c r="G1593" s="9">
+        <v>50000</v>
+      </c>
+      <c r="H1593" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1594" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1594" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1594" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1594" s="9">
+        <v>28861086</v>
+      </c>
+      <c r="D1594" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1594" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1594" s="9">
+        <v>1356</v>
+      </c>
+      <c r="G1594" s="9">
+        <v>67800</v>
+      </c>
+      <c r="H1594" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1595" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1595" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1595" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1595" s="9">
+        <v>28841781</v>
+      </c>
+      <c r="D1595" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1595" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1595" s="9">
+        <v>1356</v>
+      </c>
+      <c r="G1595" s="9">
+        <v>67800</v>
+      </c>
+      <c r="H1595" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1596" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1596" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1596" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1596" s="9">
+        <v>28865186</v>
+      </c>
+      <c r="D1596" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1596" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1596" s="9">
+        <v>1356</v>
+      </c>
+      <c r="G1596" s="9">
+        <v>67800</v>
+      </c>
+      <c r="H1596" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1597" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1597" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1597" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1597" s="9">
+        <v>28858975</v>
+      </c>
+      <c r="D1597" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1597" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1597" s="9">
+        <v>1356</v>
+      </c>
+      <c r="G1597" s="9">
+        <v>67800</v>
+      </c>
+      <c r="H1597" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1598" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1598" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1598" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1598" s="9">
+        <v>28865178</v>
+      </c>
+      <c r="D1598" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1598" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1598" s="9">
+        <v>1355</v>
+      </c>
+      <c r="G1598" s="9">
+        <v>67750</v>
+      </c>
+      <c r="H1598" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1599" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1599" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1599" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1599" s="9">
+        <v>28841500</v>
+      </c>
+      <c r="D1599" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1599" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1599" s="9">
+        <v>1356</v>
+      </c>
+      <c r="G1599" s="9">
+        <v>67800</v>
+      </c>
+      <c r="H1599" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1600" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1600" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1600" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1600" s="9">
+        <v>28863975</v>
+      </c>
+      <c r="D1600" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1600" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1600" s="9">
+        <v>1356</v>
+      </c>
+      <c r="G1600" s="9">
+        <v>67800</v>
+      </c>
+      <c r="H1600" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1601" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1601" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1601" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1601" s="9">
+        <v>28863660</v>
+      </c>
+      <c r="D1601" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1601" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1601" s="9">
+        <v>1356</v>
+      </c>
+      <c r="G1601" s="9">
+        <v>67800</v>
+      </c>
+      <c r="H1601" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1602" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1602" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1602" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1602" s="9">
+        <v>28840403</v>
+      </c>
+      <c r="D1602" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1602" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1602" s="9">
+        <v>1356</v>
+      </c>
+      <c r="G1602" s="9">
+        <v>67800</v>
+      </c>
+      <c r="H1602" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1603" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1603" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1603" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1603" s="9">
+        <v>28840379</v>
+      </c>
+      <c r="D1603" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1603" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1603" s="9">
+        <v>1356</v>
+      </c>
+      <c r="G1603" s="9">
+        <v>67800</v>
+      </c>
+      <c r="H1603" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1604" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1604" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1604" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1604" s="9">
+        <v>28814572</v>
+      </c>
+      <c r="D1604" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1604" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1604" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1604" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1604" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1605" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1605" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1605" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1605" s="9">
+        <v>28345700</v>
+      </c>
+      <c r="D1605" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1605" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1605" s="9">
+        <v>1350</v>
+      </c>
+      <c r="G1605" s="9">
+        <v>67500</v>
+      </c>
+      <c r="H1605" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1606" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1606" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1606" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1606" s="9">
+        <v>28043487</v>
+      </c>
+      <c r="D1606" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1606" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1606" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1606" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1606" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1607" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1607" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1607" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1607" s="9">
+        <v>28801389</v>
+      </c>
+      <c r="D1607" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1607" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1607" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1607" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1607" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1608" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1608" s="8">
+        <v>46161</v>
+      </c>
+      <c r="B1608" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1608" s="9">
+        <v>28060267</v>
+      </c>
+      <c r="D1608" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1608" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="F1608" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1608" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1608" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1609" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1609" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1609" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1609" s="6">
+        <v>28040236</v>
+      </c>
+      <c r="D1609" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1609" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="F1609" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1609" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1609" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1610" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1610" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1610" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1610" s="6">
+        <v>29001401</v>
+      </c>
+      <c r="D1610" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1610" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="F1610" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1610" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1610" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1611" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1611" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1611" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1611" s="6">
+        <v>28077717</v>
+      </c>
+      <c r="D1611" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1611" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="F1611" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1611" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1611" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1612" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1612" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1612" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1612" s="6">
+        <v>29145489</v>
+      </c>
+      <c r="D1612" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1612" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="F1612" s="6">
+        <v>1300</v>
+      </c>
+      <c r="G1612" s="6">
+        <v>65000</v>
+      </c>
+      <c r="H1612" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1613" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1613" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1613" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1613" s="6">
+        <v>87817599</v>
+      </c>
+      <c r="D1613" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1613" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="F1613" s="6">
+        <v>980</v>
+      </c>
+      <c r="G1613" s="6">
+        <v>49000</v>
+      </c>
+      <c r="H1613" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1614" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1614" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1614" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1614" s="6">
+        <v>91901645</v>
+      </c>
+      <c r="D1614" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1614" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="F1614" s="6">
+        <v>1000</v>
+      </c>
+      <c r="G1614" s="6">
+        <v>50000</v>
+      </c>
+      <c r="H1614" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1615" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1615" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1615" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1615" s="6">
+        <v>87782181</v>
+      </c>
+      <c r="D1615" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1615" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="F1615" s="6">
+        <v>900</v>
+      </c>
+      <c r="G1615" s="6">
+        <v>45000</v>
+      </c>
+      <c r="H1615" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1616" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1616" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1616" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1616" s="6">
+        <v>28873560</v>
+      </c>
+      <c r="D1616" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1616" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1616" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1616" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1616" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1617" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1617" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1617" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1617" s="6">
+        <v>29026663</v>
+      </c>
+      <c r="D1617" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1617" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1617" s="6">
+        <v>1340</v>
+      </c>
+      <c r="G1617" s="6">
+        <v>67000</v>
+      </c>
+      <c r="H1617" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1618" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1618" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1618" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1618" s="6">
+        <v>28865632</v>
+      </c>
+      <c r="D1618" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1618" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1618" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1618" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1618" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1619" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1619" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1619" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1619" s="6">
+        <v>29222635</v>
+      </c>
+      <c r="D1619" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1619" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1619" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1619" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1619" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1620" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1620" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1620" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1620" s="6">
+        <v>29222627</v>
+      </c>
+      <c r="D1620" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1620" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1620" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1620" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1620" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1621" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1621" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1621" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1621" s="6">
+        <v>28840916</v>
+      </c>
+      <c r="D1621" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1621" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1621" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1621" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1621" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1622" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1622" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1622" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1622" s="6">
+        <v>28841401</v>
+      </c>
+      <c r="D1622" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1622" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1622" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1622" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1622" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1623" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1623" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1623" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1623" s="6">
+        <v>29305216</v>
+      </c>
+      <c r="D1623" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1623" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F1623" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1623" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1623" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1624" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1624" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1624" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1624" s="6">
+        <v>29452521</v>
+      </c>
+      <c r="D1624" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1624" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F1624" s="6">
+        <v>1355</v>
+      </c>
+      <c r="G1624" s="6">
+        <v>67750</v>
+      </c>
+      <c r="H1624" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1625" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1625" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1625" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1625" s="6">
+        <v>29452232</v>
+      </c>
+      <c r="D1625" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1625" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F1625" s="6">
+        <v>1354</v>
+      </c>
+      <c r="G1625" s="6">
+        <v>67700</v>
+      </c>
+      <c r="H1625" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1626" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1626" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1626" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1626" s="6">
+        <v>28044477</v>
+      </c>
+      <c r="D1626" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1626" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1626" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1626" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1626" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1627" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1627" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1627" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1627" s="6">
+        <v>28053445</v>
+      </c>
+      <c r="D1627" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1627" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1627" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1627" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1627" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1628" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1628" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1628" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1628" s="6">
+        <v>28814523</v>
+      </c>
+      <c r="D1628" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1628" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1628" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1628" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1628" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1629" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1629" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1629" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1629" s="6">
+        <v>28289395</v>
+      </c>
+      <c r="D1629" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1629" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1629" s="6">
+        <v>1340</v>
+      </c>
+      <c r="G1629" s="6">
+        <v>67000</v>
+      </c>
+      <c r="H1629" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1630" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1630" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1630" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1630" s="6">
+        <v>28015352</v>
+      </c>
+      <c r="D1630" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1630" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1630" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1630" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1630" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1631" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1631" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1631" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1631" s="6">
+        <v>28010403</v>
+      </c>
+      <c r="D1631" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1631" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="F1631" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1631" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1631" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1632" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1632" s="5">
+        <v>46162</v>
+      </c>
+      <c r="B1632" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1632" s="6">
+        <v>28010775</v>
+      </c>
+      <c r="D1632" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1632" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="F1632" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1632" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1632" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1633" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1633" s="8">
+        <v>46162</v>
+      </c>
+      <c r="B1633" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1633" s="9">
+        <v>28347201</v>
+      </c>
+      <c r="D1633" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1633" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F1633" s="9">
+        <v>1257</v>
+      </c>
+      <c r="G1633" s="9">
+        <v>62850</v>
+      </c>
+      <c r="H1633" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1634" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1634" s="8">
+        <v>46162</v>
+      </c>
+      <c r="B1634" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1634" s="9">
+        <v>98215205</v>
+      </c>
+      <c r="D1634" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1634" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F1634" s="9">
+        <v>1190</v>
+      </c>
+      <c r="G1634" s="9">
+        <v>68530</v>
+      </c>
+      <c r="H1634" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1635" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1635" s="8">
+        <v>46162</v>
+      </c>
+      <c r="B1635" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1635" s="9">
+        <v>98219306</v>
+      </c>
+      <c r="D1635" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1635" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F1635" s="9">
+        <v>1170</v>
+      </c>
+      <c r="G1635" s="9">
+        <v>70360</v>
+      </c>
+      <c r="H1635" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1636" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1636" s="8">
+        <v>46162</v>
+      </c>
+      <c r="B1636" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1636" s="9">
+        <v>99409310</v>
+      </c>
+      <c r="D1636" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1636" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F1636" s="9">
+        <v>1197</v>
+      </c>
+      <c r="G1636" s="9">
+        <v>68320</v>
+      </c>
+      <c r="H1636" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1637" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1637" s="8">
+        <v>46162</v>
+      </c>
+      <c r="B1637" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1637" s="9">
+        <v>28841153</v>
+      </c>
+      <c r="D1637" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1637" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1637" s="9">
+        <v>1356</v>
+      </c>
+      <c r="G1637" s="9">
+        <v>67800</v>
+      </c>
+      <c r="H1637" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1638" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1638" s="8">
+        <v>46162</v>
+      </c>
+      <c r="B1638" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1638" s="9">
+        <v>28840437</v>
+      </c>
+      <c r="D1638" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1638" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1638" s="9">
+        <v>1356</v>
+      </c>
+      <c r="G1638" s="9">
+        <v>67800</v>
+      </c>
+      <c r="H1638" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1639" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1639" s="8">
+        <v>46162</v>
+      </c>
+      <c r="B1639" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1639" s="9">
+        <v>28863512</v>
+      </c>
+      <c r="D1639" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1639" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1639" s="9">
+        <v>1356</v>
+      </c>
+      <c r="G1639" s="9">
+        <v>67800</v>
+      </c>
+      <c r="H1639" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1640" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1640" s="8">
+        <v>46162</v>
+      </c>
+      <c r="B1640" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1640" s="9">
+        <v>28090983</v>
+      </c>
+      <c r="D1640" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1640" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1640" s="9">
+        <v>1356</v>
+      </c>
+      <c r="G1640" s="9">
+        <v>67800</v>
+      </c>
+      <c r="H1640" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1641" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1641" s="8">
+        <v>46163</v>
+      </c>
+      <c r="B1641" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1641" s="9">
+        <v>91901637</v>
+      </c>
+      <c r="D1641" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1641" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1641" s="9">
+        <v>1000</v>
+      </c>
+      <c r="G1641" s="9">
+        <v>50000</v>
+      </c>
+      <c r="H1641" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1642" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1642" s="8">
+        <v>46163</v>
+      </c>
+      <c r="B1642" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1642" s="9">
+        <v>91901652</v>
+      </c>
+      <c r="D1642" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1642" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1642" s="9">
+        <v>1000</v>
+      </c>
+      <c r="G1642" s="9">
+        <v>50000</v>
+      </c>
+      <c r="H1642" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1643" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1643" s="8">
+        <v>46163</v>
+      </c>
+      <c r="B1643" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1643" s="9">
+        <v>91913160</v>
+      </c>
+      <c r="D1643" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1643" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1643" s="9">
+        <v>1000</v>
+      </c>
+      <c r="G1643" s="9">
+        <v>50000</v>
+      </c>
+      <c r="H1643" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1644" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1644" s="8">
+        <v>46163</v>
+      </c>
+      <c r="B1644" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1644" s="9">
+        <v>28040756</v>
+      </c>
+      <c r="D1644" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1644" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1644" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1644" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1644" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1645" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1645" s="8">
+        <v>46163</v>
+      </c>
+      <c r="B1645" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1645" s="9">
+        <v>28054153</v>
+      </c>
+      <c r="D1645" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1645" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1645" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1645" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1645" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1646" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1646" s="8">
+        <v>46163</v>
+      </c>
+      <c r="B1646" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1646" s="9">
+        <v>28820116</v>
+      </c>
+      <c r="D1646" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1646" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1646" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1646" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1646" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1647" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1647" s="8">
+        <v>46163</v>
+      </c>
+      <c r="B1647" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1647" s="9">
+        <v>28021756</v>
+      </c>
+      <c r="D1647" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1647" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1647" s="9">
+        <v>1358</v>
+      </c>
+      <c r="G1647" s="9">
+        <v>67900</v>
+      </c>
+      <c r="H1647" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1648" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1648" s="8">
+        <v>46163</v>
+      </c>
+      <c r="B1648" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1648" s="9">
+        <v>28011559</v>
+      </c>
+      <c r="D1648" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1648" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1648" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1648" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1648" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1649" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1649" s="8">
+        <v>46163</v>
+      </c>
+      <c r="B1649" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1649" s="9">
+        <v>28821551</v>
+      </c>
+      <c r="D1649" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1649" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1649" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1649" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1649" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1650" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1650" s="8">
+        <v>46163</v>
+      </c>
+      <c r="B1650" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1650" s="9">
+        <v>28010569</v>
+      </c>
+      <c r="D1650" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1650" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1650" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1650" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1650" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1651" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1651" s="8">
+        <v>46163</v>
+      </c>
+      <c r="B1651" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1651" s="9">
+        <v>29109477</v>
+      </c>
+      <c r="D1651" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1651" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="F1651" s="9">
+        <v>1336</v>
+      </c>
+      <c r="G1651" s="9">
+        <v>66800</v>
+      </c>
+      <c r="H1651" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1652" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1652" s="8">
+        <v>46163</v>
+      </c>
+      <c r="B1652" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1652" s="9">
+        <v>29900198</v>
+      </c>
+      <c r="D1652" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1652" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="F1652" s="9">
+        <v>1339</v>
+      </c>
+      <c r="G1652" s="9">
+        <v>66950</v>
+      </c>
+      <c r="H1652" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1653" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1653" s="8">
+        <v>46163</v>
+      </c>
+      <c r="B1653" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1653" s="9">
+        <v>28345403</v>
+      </c>
+      <c r="D1653" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1653" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F1653" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1653" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1653" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1654" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1654" s="8">
+        <v>46163</v>
+      </c>
+      <c r="B1654" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1654" s="9">
+        <v>28815173</v>
+      </c>
+      <c r="D1654" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1654" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F1654" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1654" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1654" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1655" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1655" s="8">
+        <v>46164</v>
+      </c>
+      <c r="B1655" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1655" s="9">
+        <v>29140340</v>
+      </c>
+      <c r="D1655" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1655" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1655" s="9">
+        <v>1336</v>
+      </c>
+      <c r="G1655" s="9">
+        <v>66800</v>
+      </c>
+      <c r="H1655" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1656" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1656" s="8">
+        <v>46164</v>
+      </c>
+      <c r="B1656" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1656" s="9">
+        <v>28022754</v>
+      </c>
+      <c r="D1656" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1656" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1656" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1656" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1656" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1657" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1657" s="8">
+        <v>46164</v>
+      </c>
+      <c r="B1657" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1657" s="9">
+        <v>28808046</v>
+      </c>
+      <c r="D1657" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1657" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1657" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1657" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1657" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1658" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1658" s="8">
+        <v>46164</v>
+      </c>
+      <c r="B1658" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1658" s="9">
+        <v>28051902</v>
+      </c>
+      <c r="D1658" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1658" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1658" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1658" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1658" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1659" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1659" s="8">
+        <v>46164</v>
+      </c>
+      <c r="B1659" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1659" s="9">
+        <v>28051621</v>
+      </c>
+      <c r="D1659" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1659" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1659" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1659" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1659" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1660" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1660" s="8">
+        <v>46164</v>
+      </c>
+      <c r="B1660" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1660" s="9">
+        <v>28023745</v>
+      </c>
+      <c r="D1660" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1660" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1660" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1660" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1660" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1661" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1661" s="8">
+        <v>46164</v>
+      </c>
+      <c r="B1661" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1661" s="9">
+        <v>28047389</v>
+      </c>
+      <c r="D1661" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1661" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="F1661" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1661" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1661" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1662" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1662" s="8">
+        <v>46164</v>
+      </c>
+      <c r="B1662" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1662" s="9">
+        <v>28346229</v>
+      </c>
+      <c r="D1662" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1662" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="F1662" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1662" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1662" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1663" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1663" s="8">
+        <v>46164</v>
+      </c>
+      <c r="B1663" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1663" s="9">
+        <v>28012318</v>
+      </c>
+      <c r="D1663" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1663" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="F1663" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1663" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1663" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1664" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1664" s="8">
+        <v>46164</v>
+      </c>
+      <c r="B1664" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1664" s="9">
+        <v>28045664</v>
+      </c>
+      <c r="D1664" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1664" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="F1664" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1664" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1664" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1665" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1665" s="8">
+        <v>46164</v>
+      </c>
+      <c r="B1665" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1665" s="9">
+        <v>28045151</v>
+      </c>
+      <c r="D1665" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1665" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="F1665" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1665" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1665" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1666" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1666" s="8">
+        <v>46164</v>
+      </c>
+      <c r="B1666" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1666" s="9">
+        <v>24671455</v>
+      </c>
+      <c r="D1666" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1666" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="F1666" s="9">
+        <v>1210</v>
+      </c>
+      <c r="G1666" s="9">
+        <v>60500</v>
+      </c>
+      <c r="H1666" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1667" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1667" s="8">
+        <v>46164</v>
+      </c>
+      <c r="B1667" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1667" s="9">
+        <v>28348522</v>
+      </c>
+      <c r="D1667" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1667" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F1667" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1667" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1667" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1668" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1668" s="8">
+        <v>46164</v>
+      </c>
+      <c r="B1668" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1668" s="9">
+        <v>28801306</v>
+      </c>
+      <c r="D1668" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1668" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1668" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1668" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1668" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1669" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1669" s="8">
+        <v>46164</v>
+      </c>
+      <c r="B1669" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1669" s="9">
+        <v>28025344</v>
+      </c>
+      <c r="D1669" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="E1669" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1669" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1669" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1669" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1670" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1670" s="8">
+        <v>46164</v>
+      </c>
+      <c r="B1670" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1670" s="9">
+        <v>28059061</v>
+      </c>
+      <c r="D1670" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="E1670" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1670" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1670" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1670" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1671" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1671" s="8">
+        <v>46164</v>
+      </c>
+      <c r="B1671" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1671" s="9">
+        <v>28818904</v>
+      </c>
+      <c r="D1671" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="E1671" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1671" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1671" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1671" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1672" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1672" s="8">
+        <v>46164</v>
+      </c>
+      <c r="B1672" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1672" s="9">
+        <v>28801546</v>
+      </c>
+      <c r="D1672" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="E1672" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F1672" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1672" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1672" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1673" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1673" s="8">
+        <v>46165</v>
+      </c>
+      <c r="B1673" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1673" s="9">
+        <v>28887750</v>
+      </c>
+      <c r="D1673" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1673" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1673" s="9">
+        <v>1356</v>
+      </c>
+      <c r="G1673" s="9">
+        <v>67800</v>
+      </c>
+      <c r="H1673" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1674" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1674" s="8">
+        <v>46165</v>
+      </c>
+      <c r="B1674" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1674" s="9">
+        <v>29445285</v>
+      </c>
+      <c r="D1674" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1674" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1674" s="9">
+        <v>1356</v>
+      </c>
+      <c r="G1674" s="9">
+        <v>67800</v>
+      </c>
+      <c r="H1674" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1675" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1675" s="8">
+        <v>46165</v>
+      </c>
+      <c r="B1675" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1675" s="9">
+        <v>29238540</v>
+      </c>
+      <c r="D1675" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1675" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1675" s="9">
+        <v>1356</v>
+      </c>
+      <c r="G1675" s="9">
+        <v>67800</v>
+      </c>
+      <c r="H1675" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1676" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1676" s="8">
+        <v>46165</v>
+      </c>
+      <c r="B1676" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1676" s="9">
+        <v>28351336</v>
+      </c>
+      <c r="D1676" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1676" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1676" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1676" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1676" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1677" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1677" s="8">
+        <v>46165</v>
+      </c>
+      <c r="B1677" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1677" s="9">
+        <v>23539950</v>
+      </c>
+      <c r="D1677" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1677" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1677" s="9">
+        <v>1320</v>
+      </c>
+      <c r="G1677" s="9">
+        <v>66000</v>
+      </c>
+      <c r="H1677" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1678" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1678" s="8">
+        <v>46165</v>
+      </c>
+      <c r="B1678" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1678" s="9">
+        <v>24343063</v>
+      </c>
+      <c r="D1678" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1678" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1678" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1678" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1678" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1679" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1679" s="8">
+        <v>46165</v>
+      </c>
+      <c r="B1679" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1679" s="9">
+        <v>26230490</v>
+      </c>
+      <c r="D1679" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1679" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1679" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1679" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1679" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1680" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1680" s="8">
+        <v>46165</v>
+      </c>
+      <c r="B1680" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1680" s="9">
+        <v>24425761</v>
+      </c>
+      <c r="D1680" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1680" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1680" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1680" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1680" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1681" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1681" s="8">
+        <v>46165</v>
+      </c>
+      <c r="B1681" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1681" s="9">
+        <v>91916502</v>
+      </c>
+      <c r="D1681" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1681" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1681" s="9">
+        <v>1000</v>
+      </c>
+      <c r="G1681" s="9">
+        <v>50000</v>
+      </c>
+      <c r="H1681" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1682" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1682" s="8">
+        <v>46165</v>
+      </c>
+      <c r="B1682" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1682" s="9">
+        <v>87782157</v>
+      </c>
+      <c r="D1682" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1682" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1682" s="9">
+        <v>900</v>
+      </c>
+      <c r="G1682" s="9">
+        <v>45000</v>
+      </c>
+      <c r="H1682" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1683" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1683" s="8">
+        <v>46165</v>
+      </c>
+      <c r="B1683" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1683" s="9">
+        <v>87795795</v>
+      </c>
+      <c r="D1683" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1683" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="F1683" s="9">
+        <v>900</v>
+      </c>
+      <c r="G1683" s="9">
+        <v>45000</v>
+      </c>
+      <c r="H1683" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1684" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1684" s="8">
+        <v>46165</v>
+      </c>
+      <c r="B1684" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1684" s="9">
+        <v>91916486</v>
+      </c>
+      <c r="D1684" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1684" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1684" s="9">
+        <v>920</v>
+      </c>
+      <c r="G1684" s="9">
+        <v>46000</v>
+      </c>
+      <c r="H1684" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1685" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1685" s="8">
+        <v>46165</v>
+      </c>
+      <c r="B1685" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1685" s="9">
+        <v>23546906</v>
+      </c>
+      <c r="D1685" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1685" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1685" s="9">
+        <v>1280</v>
+      </c>
+      <c r="G1685" s="9">
+        <v>64000</v>
+      </c>
+      <c r="H1685" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1686" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1686" s="8">
+        <v>46165</v>
+      </c>
+      <c r="B1686" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1686" s="9">
+        <v>23470958</v>
+      </c>
+      <c r="D1686" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1686" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1686" s="9">
+        <v>1280</v>
+      </c>
+      <c r="G1686" s="9">
+        <v>64000</v>
+      </c>
+      <c r="H1686" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1687" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1687" s="8">
+        <v>46165</v>
+      </c>
+      <c r="B1687" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1687" s="9">
+        <v>28029346</v>
+      </c>
+      <c r="D1687" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1687" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1687" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1687" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1687" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1688" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1688" s="8">
+        <v>46165</v>
+      </c>
+      <c r="B1688" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1688" s="9">
+        <v>24425852</v>
+      </c>
+      <c r="D1688" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1688" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1688" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1688" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1688" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1689" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1689" s="8">
+        <v>46165</v>
+      </c>
+      <c r="B1689" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1689" s="9">
+        <v>28066751</v>
+      </c>
+      <c r="D1689" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1689" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1689" s="9">
+        <v>1300</v>
+      </c>
+      <c r="G1689" s="9">
+        <v>65000</v>
+      </c>
+      <c r="H1689" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1690" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1690" s="8">
+        <v>46165</v>
+      </c>
+      <c r="B1690" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1690" s="9">
+        <v>52460466</v>
+      </c>
+      <c r="D1690" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1690" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1690" s="9">
+        <v>1360</v>
+      </c>
+      <c r="G1690" s="9">
+        <v>68000</v>
+      </c>
+      <c r="H1690" s="10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1691" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1691" s="5">
+        <v>46165</v>
+      </c>
+      <c r="B1691" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1691" s="6">
+        <v>28848133</v>
+      </c>
+      <c r="D1691" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1691" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1691" s="6">
+        <v>1359</v>
+      </c>
+      <c r="G1691" s="6">
+        <v>67950</v>
+      </c>
+      <c r="H1691" s="7"/>
+    </row>
+    <row r="1692" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1692" s="5">
+        <v>46165</v>
+      </c>
+      <c r="B1692" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1692" s="6">
+        <v>28090264</v>
+      </c>
+      <c r="D1692" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1692" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1692" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1692" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1692" s="7"/>
+    </row>
+    <row r="1693" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1693" s="5">
+        <v>46165</v>
+      </c>
+      <c r="B1693" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1693" s="6">
+        <v>28090785</v>
+      </c>
+      <c r="D1693" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1693" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1693" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1693" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1693" s="7"/>
+    </row>
+    <row r="1694" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1694" s="5">
+        <v>46165</v>
+      </c>
+      <c r="B1694" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1694" s="6">
+        <v>28847770</v>
+      </c>
+      <c r="D1694" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1694" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1694" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1694" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1694" s="7"/>
+    </row>
+    <row r="1695" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1695" s="5">
+        <v>46165</v>
+      </c>
+      <c r="B1695" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1695" s="6">
+        <v>28846830</v>
+      </c>
+      <c r="D1695" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1695" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1695" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1695" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1695" s="7"/>
+    </row>
+    <row r="1696" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1696" s="5">
+        <v>46166</v>
+      </c>
+      <c r="B1696" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1696" s="6">
+        <v>29021144</v>
+      </c>
+      <c r="D1696" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1696" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1696" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1696" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1696" s="7"/>
+    </row>
+    <row r="1697" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1697" s="5">
+        <v>46166</v>
+      </c>
+      <c r="B1697" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1697" s="6">
+        <v>28002517</v>
+      </c>
+      <c r="D1697" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1697" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1697" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1697" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1697" s="7"/>
+    </row>
+    <row r="1698" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1698" s="5">
+        <v>46166</v>
+      </c>
+      <c r="B1698" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1698" s="6">
+        <v>29840592</v>
+      </c>
+      <c r="D1698" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1698" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1698" s="6">
+        <v>1340</v>
+      </c>
+      <c r="G1698" s="6">
+        <v>67000</v>
+      </c>
+      <c r="H1698" s="7"/>
+    </row>
+    <row r="1699" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1699" s="5">
+        <v>46166</v>
+      </c>
+      <c r="B1699" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1699" s="6">
+        <v>28855153</v>
+      </c>
+      <c r="D1699" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1699" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1699" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1699" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1699" s="7"/>
+    </row>
+    <row r="1700" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1700" s="5">
+        <v>46166</v>
+      </c>
+      <c r="B1700" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1700" s="6">
+        <v>28856086</v>
+      </c>
+      <c r="D1700" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1700" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1700" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1700" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1700" s="7"/>
+    </row>
+    <row r="1701" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1701" s="5">
+        <v>46166</v>
+      </c>
+      <c r="B1701" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1701" s="6">
+        <v>28854131</v>
+      </c>
+      <c r="D1701" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1701" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1701" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1701" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1701" s="7"/>
+    </row>
+    <row r="1702" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1702" s="5">
+        <v>46166</v>
+      </c>
+      <c r="B1702" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1702" s="6">
+        <v>28856144</v>
+      </c>
+      <c r="D1702" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1702" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1702" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1702" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1702" s="7"/>
+    </row>
+    <row r="1703" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1703" s="5">
+        <v>46166</v>
+      </c>
+      <c r="B1703" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1703" s="6">
+        <v>28856029</v>
+      </c>
+      <c r="D1703" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1703" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1703" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1703" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1703" s="7"/>
+    </row>
+    <row r="1704" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1704" s="5">
+        <v>46167</v>
+      </c>
+      <c r="B1704" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1704" s="6">
+        <v>29221074</v>
+      </c>
+      <c r="D1704" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1704" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1704" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1704" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1704" s="7"/>
+    </row>
+    <row r="1705" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1705" s="5">
+        <v>46167</v>
+      </c>
+      <c r="B1705" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1705" s="6">
+        <v>29410305</v>
+      </c>
+      <c r="D1705" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1705" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1705" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1705" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1705" s="7"/>
+    </row>
+    <row r="1706" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1706" s="5">
+        <v>46167</v>
+      </c>
+      <c r="B1706" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1706" s="6">
+        <v>29135431</v>
+      </c>
+      <c r="D1706" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1706" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1706" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1706" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1706" s="7"/>
+    </row>
+    <row r="1707" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1707" s="5">
+        <v>46167</v>
+      </c>
+      <c r="B1707" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1707" s="6">
+        <v>29221009</v>
+      </c>
+      <c r="D1707" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1707" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1707" s="6">
+        <v>1356</v>
+      </c>
+      <c r="G1707" s="6">
+        <v>67800</v>
+      </c>
+      <c r="H1707" s="7"/>
+    </row>
+    <row r="1708" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1708" s="5">
+        <v>46167</v>
+      </c>
+      <c r="B1708" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1708" s="6">
+        <v>28819480</v>
+      </c>
+      <c r="D1708" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1708" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1708" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1708" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1708" s="7"/>
+    </row>
+    <row r="1709" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1709" s="5">
+        <v>46167</v>
+      </c>
+      <c r="B1709" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1709" s="6">
+        <v>28349660</v>
+      </c>
+      <c r="D1709" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1709" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1709" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1709" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1709" s="7"/>
+    </row>
+    <row r="1710" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1710" s="5">
+        <v>46167</v>
+      </c>
+      <c r="B1710" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1710" s="6">
+        <v>28026961</v>
+      </c>
+      <c r="D1710" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1710" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1710" s="6">
+        <v>1360</v>
+      </c>
+      <c r="G1710" s="6">
+        <v>68000</v>
+      </c>
+      <c r="H1710" s="7"/>
+    </row>
+    <row r="1711" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1711" s="8">
+        <v>46166</v>
+      </c>
+      <c r="B1711" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1711" s="9">
+        <v>91138644</v>
+      </c>
+      <c r="D1711" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1711" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F1711" s="9">
+        <v>1303</v>
+      </c>
+      <c r="G1711" s="9">
+        <v>68100</v>
+      </c>
+      <c r="H1711" s="10"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>